<commit_message>
fix(proposal_smart): v8.64 — GA 쪽별 반박 검증 결함 9건
- 상급종합병원·권역심뇌혈관 통합치료비는 그 종별 이상에서만, 종합병원 중환자실 항목은 종합병원 이상에서만
- 질병 통합치료비 수술(1-5종) : 사례 1-5종 항목으로 종 결정, 금액표 연간 1회 → 수술 1회당(약관 표 · import_dz_itc 도 수정)
- 표적 (2종및3종이상) 약물 3종이면 2종이상·3종이상 각각 지급
- 표적항암약물허가치료비Ⅲ [특정표적]/[특정면역] 배타 구분
- 수가코드 시술 치료비(하이푸 RZ566·고주파 PZ612)가 시술 단계에서 지급되도록
- 겹대괄호 세부보장 이름 읽기, 암 주요치료비 대상 범위, 사유 문구(1-7종 종·질병군·빈도)
- 회귀 7건 : carefree-40(질병 통합치료비 가입) 암·뇌 수술표만 변경, 나머지 글자 차이 0 · 이탈잘림 0
- 규칙표 105 → 107줄 · 검수표 재출력 · README v8.64

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013nQuS8bdQRpJJoVSNgEADt
</commit_message>
<xml_diff>
--- a/dist/규칙표_KCD검수결과.xlsx
+++ b/dist/규칙표_KCD검수결과.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="읽는 법" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="규칙 105개" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="규칙 107개" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="치료행위 어휘" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="질병코드 그룹표" sheetId="5" state="visible" r:id="rId5"/>
@@ -20,7 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2차 검수 · 검사비 항목" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'규칙 105개'!$A$2:$T$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'규칙 107개'!$A$2:$T$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -672,7 +672,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>메리츠 스마트 제안서 생성기 v8.63 · rules.json 의 규칙 105줄</t>
+          <t>메리츠 스마트 제안서 생성기 v8.64 · rules.json 의 규칙 107줄</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
     <row r="28" ht="17" customHeight="1">
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>규칙 105개 — 규칙표 본문. 한 줄이 규칙 하나입니다.</t>
+          <t>규칙 107개 — 규칙표 본문. 한 줄이 규칙 하나입니다.</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T107"/>
+  <dimension ref="A1:T109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2940,7 +2940,7 @@
         </is>
       </c>
       <c r="P23" s="7" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="Q23" s="10" t="inlineStr"/>
       <c r="R23" s="10" t="inlineStr">
@@ -3515,7 +3515,7 @@
         </is>
       </c>
       <c r="P31" s="7" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="Q31" s="10" t="inlineStr"/>
       <c r="R31" s="10" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>tx_target</t>
+          <t>tx_target_specific</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>표적항암약물허가치료비</t>
+          <t>표적항암약물허가치료비Ⅲ.*\[특정표적항암약물허가치료\]</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr"/>
@@ -6369,7 +6369,7 @@
       <c r="K71" s="10" t="inlineStr"/>
       <c r="L71" s="10" t="inlineStr">
         <is>
-          <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
+          <t>메모 : 통184·케336 제5조② 특정표적항암제 = 표적항암제 중 특정면역항암제를 뺀 것 — 면역·카티 치료 단계에서는 지급하지 않는다(v8.63)</t>
         </is>
       </c>
       <c r="M71" s="10" t="inlineStr">
@@ -6379,97 +6379,253 @@
       </c>
       <c r="N71" s="10" t="inlineStr">
         <is>
-          <t>표적항암약물허가치료 · 최초 1회(연간형·약물종수형은 담보명 표기대로)</t>
+          <t>특정표적항암약물허가치료(비급여 · 특정면역항암제 제외) · 최초 1회</t>
         </is>
       </c>
       <c r="O71" s="10" t="inlineStr">
         <is>
-          <t>표적항암약물허가치료비</t>
+          <t>표적항암약물허가치료비Ⅲ [특정표적] — 면역항암 단계 제외(v8.63)</t>
         </is>
       </c>
       <c r="P71" s="7" t="n">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q71" s="10" t="inlineStr"/>
       <c r="R71" s="10" t="inlineStr">
+        <is>
+          <t>갱신형 표적항암약물허가치료비Ⅲ(비급여)[특정표적항암약물허가치료]
+갱신형 계속받는 표적항암약물허가치료비Ⅲ(연간1회한)(비급여)[특정표적항암약물허가치료]
+갱신형 표적항암약물허가치료비Ⅲ(비급여)[특정표적항암약물허가치료]
+갱신형 계속받는 표적항암약물허가치료비Ⅲ(연간1회한)(비급여)[특정표적항암약물허가치료]
+갱신형표적항암약물허가치료비Ⅲ(비급여)[특정표적항암약물허가치료]</t>
+        </is>
+      </c>
+      <c r="S71" s="11" t="inlineStr"/>
+      <c r="T71" s="11" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>tx_target_immune_sub</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>표적항암약물허가치료비Ⅲ.*\[특정면역항암약물허가치료\]</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr"/>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>major_thy_skin</t>
+        </is>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H72" s="12" t="inlineStr">
+        <is>
+          <t>최초 1회</t>
+        </is>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>면역항암약물치료  (immune)</t>
+        </is>
+      </c>
+      <c r="J72" s="15" t="inlineStr"/>
+      <c r="K72" s="15" t="inlineStr"/>
+      <c r="L72" s="15" t="inlineStr">
+        <is>
+          <t>메모 : 통184·케336 제6조① 특정면역항암제 — 표적항암 단계에서는 지급하지 않는다(v8.63)</t>
+        </is>
+      </c>
+      <c r="M72" s="15" t="inlineStr">
+        <is>
+          <t>암 치료</t>
+        </is>
+      </c>
+      <c r="N72" s="15" t="inlineStr">
+        <is>
+          <t>특정면역항암약물허가치료(비급여 · 면역관문억제제·ADC·카티) · 최초 1회</t>
+        </is>
+      </c>
+      <c r="O72" s="15" t="inlineStr">
+        <is>
+          <t>표적항암약물허가치료비Ⅲ [특정면역] — 면역항암 단계에서만(v8.63)</t>
+        </is>
+      </c>
+      <c r="P72" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q72" s="15" t="inlineStr"/>
+      <c r="R72" s="15" t="inlineStr">
+        <is>
+          <t>갱신형 표적항암약물허가치료비Ⅲ(비급여)[특정면역항암약물허가치료]
+갱신형 계속받는 표적항암약물허가치료비Ⅲ(연간1회한)(비급여)[특정면역항암약물허가치료]
+갱신형 표적항암약물허가치료비Ⅲ(비급여)[특정면역항암약물허가치료]
+갱신형 계속받는 표적항암약물허가치료비Ⅲ(연간1회한)(비급여)[특정면역항암약물허가치료]
+갱신형표적항암약물허가치료비Ⅲ(비급여)[특정면역항암약물허가치료]</t>
+        </is>
+      </c>
+      <c r="S72" s="11" t="inlineStr"/>
+      <c r="T72" s="11" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>tx_target</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>표적항암약물허가치료비</t>
+        </is>
+      </c>
+      <c r="E73" s="10" t="inlineStr"/>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
+          <t>major_thy_skin</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>최초 1회</t>
+        </is>
+      </c>
+      <c r="I73" s="10" t="inlineStr">
+        <is>
+          <t>표적항암약물치료  (target)</t>
+        </is>
+      </c>
+      <c r="J73" s="10" t="inlineStr"/>
+      <c r="K73" s="10" t="inlineStr"/>
+      <c r="L73" s="10" t="inlineStr">
+        <is>
+          <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
+        </is>
+      </c>
+      <c r="M73" s="10" t="inlineStr">
+        <is>
+          <t>암 치료</t>
+        </is>
+      </c>
+      <c r="N73" s="10" t="inlineStr">
+        <is>
+          <t>표적항암약물허가치료 · 최초 1회(연간형·약물종수형은 담보명 표기대로)</t>
+        </is>
+      </c>
+      <c r="O73" s="10" t="inlineStr">
+        <is>
+          <t>표적항암약물허가치료비</t>
+        </is>
+      </c>
+      <c r="P73" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q73" s="10" t="inlineStr"/>
+      <c r="R73" s="10" t="inlineStr">
         <is>
           <t>갱신형 표적항암약물허가치료비Ⅱ
 갱신형 계속받는 표적항암약물허가치료비Ⅱ(연간1회한)
 갱신형 표적항암약물허가치료비Ⅲ(비급여)
-갱신형 표적항암약물허가치료비Ⅲ(비급여)[특정표적항암약물허가치료]
-갱신형 표적항암약물허가치료비Ⅲ(비급여)[특정면역항암약물허가치료]</t>
-        </is>
-      </c>
-      <c r="S71" s="11" t="inlineStr"/>
-      <c r="T71" s="11" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="B72" s="13" t="inlineStr">
+갱신형 계속받는 표적항암약물허가치료비Ⅲ(연간1회한)(비급여)
+갱신형 표적항암약물허가치료비(연간 약물종류 개수별)(연간1회한)[1종이상]</t>
+        </is>
+      </c>
+      <c r="S73" s="11" t="inlineStr"/>
+      <c r="T73" s="11" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>tx_immune</t>
         </is>
       </c>
-      <c r="C72" s="14" t="inlineStr">
+      <c r="C74" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D72" s="13" t="inlineStr">
+      <c r="D74" s="13" t="inlineStr">
         <is>
           <t>면역항암약물허가치료비</t>
         </is>
       </c>
-      <c r="E72" s="15" t="inlineStr"/>
-      <c r="F72" s="15" t="inlineStr">
+      <c r="E74" s="15" t="inlineStr"/>
+      <c r="F74" s="15" t="inlineStr">
         <is>
           <t>major_thy_skin</t>
         </is>
       </c>
-      <c r="G72" s="12" t="inlineStr">
+      <c r="G74" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H72" s="12" t="inlineStr">
+      <c r="H74" s="12" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I72" s="15" t="inlineStr">
+      <c r="I74" s="15" t="inlineStr">
         <is>
           <t>면역항암약물치료  (immune)</t>
         </is>
       </c>
-      <c r="J72" s="15" t="inlineStr"/>
-      <c r="K72" s="15" t="inlineStr"/>
-      <c r="L72" s="15" t="inlineStr">
+      <c r="J74" s="15" t="inlineStr"/>
+      <c r="K74" s="15" t="inlineStr"/>
+      <c r="L74" s="15" t="inlineStr">
         <is>
           <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
         </is>
       </c>
-      <c r="M72" s="15" t="inlineStr">
+      <c r="M74" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N72" s="15" t="inlineStr">
+      <c r="N74" s="15" t="inlineStr">
         <is>
           <t>비급여 면역항암약물허가치료 · 최초 1회</t>
         </is>
       </c>
-      <c r="O72" s="15" t="inlineStr">
+      <c r="O74" s="15" t="inlineStr">
         <is>
           <t>특정면역항암약물허가치료비</t>
         </is>
       </c>
-      <c r="P72" s="12" t="n">
+      <c r="P74" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="Q72" s="15" t="inlineStr"/>
-      <c r="R72" s="15" t="inlineStr">
+      <c r="Q74" s="15" t="inlineStr"/>
+      <c r="R74" s="15" t="inlineStr">
         <is>
           <t>갱신형 특정면역항암약물허가치료비
 갱신형 계속받는 특정면역항암약물허가치료비(연간1회한)
@@ -6478,76 +6634,76 @@
 갱신형 특정면역항암약물허가치료비</t>
         </is>
       </c>
-      <c r="S72" s="11" t="inlineStr"/>
-      <c r="T72" s="11" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="7" t="n">
-        <v>71</v>
-      </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="S74" s="11" t="inlineStr"/>
+      <c r="T74" s="11" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>tx_hormone</t>
         </is>
       </c>
-      <c r="C73" s="9" t="inlineStr">
+      <c r="C75" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D73" s="8" t="inlineStr">
+      <c r="D75" s="8" t="inlineStr">
         <is>
           <t>호르몬약물허가치료비</t>
         </is>
       </c>
-      <c r="E73" s="10" t="inlineStr"/>
-      <c r="F73" s="10" t="inlineStr">
+      <c r="E75" s="10" t="inlineStr"/>
+      <c r="F75" s="10" t="inlineStr">
         <is>
           <t>암 또는 유사암</t>
         </is>
       </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="G75" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H73" s="7" t="inlineStr">
+      <c r="H75" s="7" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I73" s="10" t="inlineStr">
+      <c r="I75" s="10" t="inlineStr">
         <is>
           <t>항암 호르몬약물치료  (hormone)</t>
         </is>
       </c>
-      <c r="J73" s="10" t="inlineStr"/>
-      <c r="K73" s="10" t="inlineStr"/>
-      <c r="L73" s="10" t="inlineStr">
+      <c r="J75" s="10" t="inlineStr"/>
+      <c r="K75" s="10" t="inlineStr"/>
+      <c r="L75" s="10" t="inlineStr">
         <is>
           <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
         </is>
       </c>
-      <c r="M73" s="10" t="inlineStr">
+      <c r="M75" s="10" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N73" s="10" t="inlineStr">
+      <c r="N75" s="10" t="inlineStr">
         <is>
           <t>항암 호르몬약물 · 최초 1회</t>
         </is>
       </c>
-      <c r="O73" s="10" t="inlineStr">
+      <c r="O75" s="10" t="inlineStr">
         <is>
           <t>항암 호르몬약물치료비</t>
         </is>
       </c>
-      <c r="P73" s="7" t="n">
+      <c r="P75" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="Q73" s="10" t="inlineStr"/>
-      <c r="R73" s="10" t="inlineStr">
+      <c r="Q75" s="10" t="inlineStr"/>
+      <c r="R75" s="10" t="inlineStr">
         <is>
           <t>특정호르몬약물허가치료비
 특정항암호르몬약물허가치료비
@@ -6556,76 +6712,76 @@
 특정호르몬약물허가치료비 (감액및면책기간미적용)</t>
         </is>
       </c>
-      <c r="S73" s="11" t="inlineStr"/>
-      <c r="T73" s="11" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="12" t="n">
-        <v>72</v>
-      </c>
-      <c r="B74" s="13" t="inlineStr">
+      <c r="S75" s="11" t="inlineStr"/>
+      <c r="T75" s="11" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" s="13" t="inlineStr">
         <is>
           <t>tx_imrt</t>
         </is>
       </c>
-      <c r="C74" s="14" t="inlineStr">
+      <c r="C76" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D76" s="13" t="inlineStr">
         <is>
           <t>항암세기조절방사선치료비</t>
         </is>
       </c>
-      <c r="E74" s="15" t="inlineStr"/>
-      <c r="F74" s="15" t="inlineStr">
+      <c r="E76" s="15" t="inlineStr"/>
+      <c r="F76" s="15" t="inlineStr">
         <is>
           <t>major_thy_skin</t>
         </is>
       </c>
-      <c r="G74" s="12" t="inlineStr">
+      <c r="G76" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H74" s="12" t="inlineStr">
+      <c r="H76" s="12" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I74" s="15" t="inlineStr">
+      <c r="I76" s="15" t="inlineStr">
         <is>
           <t>세기조절방사선치료(IMRT)  (imrt)</t>
         </is>
       </c>
-      <c r="J74" s="15" t="inlineStr"/>
-      <c r="K74" s="15" t="inlineStr"/>
-      <c r="L74" s="15" t="inlineStr">
+      <c r="J76" s="15" t="inlineStr"/>
+      <c r="K76" s="15" t="inlineStr"/>
+      <c r="L76" s="15" t="inlineStr">
         <is>
           <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
         </is>
       </c>
-      <c r="M74" s="15" t="inlineStr">
+      <c r="M76" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N74" s="15" t="inlineStr">
+      <c r="N76" s="15" t="inlineStr">
         <is>
           <t>세기조절방사선치료 · 최초 1회</t>
         </is>
       </c>
-      <c r="O74" s="15" t="inlineStr">
+      <c r="O76" s="15" t="inlineStr">
         <is>
           <t>항암세기조절방사선치료비</t>
         </is>
       </c>
-      <c r="P74" s="12" t="n">
+      <c r="P76" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="Q74" s="15" t="inlineStr"/>
-      <c r="R74" s="15" t="inlineStr">
+      <c r="Q76" s="15" t="inlineStr"/>
+      <c r="R76" s="15" t="inlineStr">
         <is>
           <t>갱신형 항암세기조절방사선치료비
 갱신형 항암세기조절방사선치료비 (감액및면책기간미적용)
@@ -6634,76 +6790,76 @@
 갱신형항암세기조절방사선치료비</t>
         </is>
       </c>
-      <c r="S74" s="11" t="inlineStr"/>
-      <c r="T74" s="11" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="7" t="n">
-        <v>73</v>
-      </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="S76" s="11" t="inlineStr"/>
+      <c r="T76" s="11" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>tx_proton</t>
         </is>
       </c>
-      <c r="C75" s="9" t="inlineStr">
+      <c r="C77" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D75" s="8" t="inlineStr">
+      <c r="D77" s="8" t="inlineStr">
         <is>
           <t>항암양성자방사선치료비</t>
         </is>
       </c>
-      <c r="E75" s="10" t="inlineStr"/>
-      <c r="F75" s="10" t="inlineStr">
+      <c r="E77" s="10" t="inlineStr"/>
+      <c r="F77" s="10" t="inlineStr">
         <is>
           <t>major_thy_skin</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="G77" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H75" s="7" t="inlineStr">
+      <c r="H77" s="7" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I75" s="10" t="inlineStr">
+      <c r="I77" s="10" t="inlineStr">
         <is>
           <t>양성자 방사선치료  (proton)</t>
         </is>
       </c>
-      <c r="J75" s="10" t="inlineStr"/>
-      <c r="K75" s="10" t="inlineStr"/>
-      <c r="L75" s="10" t="inlineStr">
+      <c r="J77" s="10" t="inlineStr"/>
+      <c r="K77" s="10" t="inlineStr"/>
+      <c r="L77" s="10" t="inlineStr">
         <is>
           <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
         </is>
       </c>
-      <c r="M75" s="10" t="inlineStr">
+      <c r="M77" s="10" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N75" s="10" t="inlineStr">
+      <c r="N77" s="10" t="inlineStr">
         <is>
           <t>양성자방사선치료 · 최초 1회</t>
         </is>
       </c>
-      <c r="O75" s="10" t="inlineStr">
+      <c r="O77" s="10" t="inlineStr">
         <is>
           <t>항암양성자방사선치료비</t>
         </is>
       </c>
-      <c r="P75" s="7" t="n">
+      <c r="P77" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="Q75" s="10" t="inlineStr"/>
-      <c r="R75" s="10" t="inlineStr">
+      <c r="Q77" s="10" t="inlineStr"/>
+      <c r="R77" s="10" t="inlineStr">
         <is>
           <t>갱신형 항암양성자방사선치료비
 갱신형 항암양성자방사선치료비 (감액및면책기간미적용)
@@ -6712,76 +6868,76 @@
 갱신형항암양성자방사선치료비</t>
         </is>
       </c>
-      <c r="S75" s="11" t="inlineStr"/>
-      <c r="T75" s="11" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="12" t="n">
-        <v>74</v>
-      </c>
-      <c r="B76" s="13" t="inlineStr">
+      <c r="S77" s="11" t="inlineStr"/>
+      <c r="T77" s="11" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
         <is>
           <t>tx_carbon</t>
         </is>
       </c>
-      <c r="C76" s="14" t="inlineStr">
+      <c r="C78" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D76" s="13" t="inlineStr">
+      <c r="D78" s="13" t="inlineStr">
         <is>
           <t>항암중입자방사선치료비</t>
         </is>
       </c>
-      <c r="E76" s="15" t="inlineStr"/>
-      <c r="F76" s="15" t="inlineStr">
+      <c r="E78" s="15" t="inlineStr"/>
+      <c r="F78" s="15" t="inlineStr">
         <is>
           <t>major_thy_skin</t>
         </is>
       </c>
-      <c r="G76" s="12" t="inlineStr">
+      <c r="G78" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H76" s="12" t="inlineStr">
+      <c r="H78" s="12" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I76" s="15" t="inlineStr">
+      <c r="I78" s="15" t="inlineStr">
         <is>
           <t>중입자 방사선치료  (carbon)</t>
         </is>
       </c>
-      <c r="J76" s="15" t="inlineStr"/>
-      <c r="K76" s="15" t="inlineStr"/>
-      <c r="L76" s="15" t="inlineStr">
+      <c r="J78" s="15" t="inlineStr"/>
+      <c r="K78" s="15" t="inlineStr"/>
+      <c r="L78" s="15" t="inlineStr">
         <is>
           <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
         </is>
       </c>
-      <c r="M76" s="15" t="inlineStr">
+      <c r="M78" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N76" s="15" t="inlineStr">
+      <c r="N78" s="15" t="inlineStr">
         <is>
           <t>중입자방사선치료 · 최초 1회</t>
         </is>
       </c>
-      <c r="O76" s="15" t="inlineStr">
+      <c r="O78" s="15" t="inlineStr">
         <is>
           <t>항암중입자방사선치료비</t>
         </is>
       </c>
-      <c r="P76" s="12" t="n">
+      <c r="P78" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="Q76" s="15" t="inlineStr"/>
-      <c r="R76" s="15" t="inlineStr">
+      <c r="Q78" s="15" t="inlineStr"/>
+      <c r="R78" s="15" t="inlineStr">
         <is>
           <t>항암중입자방사선치료비
 항암중입자방사선치료비 (감액및면책기간미적용)
@@ -6790,72 +6946,72 @@
 항암중입자방사선치료비</t>
         </is>
       </c>
-      <c r="S76" s="11" t="inlineStr"/>
-      <c r="T76" s="11" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="7" t="n">
-        <v>75</v>
-      </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="S78" s="11" t="inlineStr"/>
+      <c r="T78" s="11" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
         <is>
           <t>tx_robot</t>
         </is>
       </c>
-      <c r="C77" s="9" t="inlineStr">
+      <c r="C79" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D77" s="8" t="inlineStr">
+      <c r="D79" s="8" t="inlineStr">
         <is>
           <t>다빈치로봇</t>
         </is>
       </c>
-      <c r="E77" s="10" t="inlineStr"/>
-      <c r="F77" s="10" t="inlineStr">
+      <c r="E79" s="10" t="inlineStr"/>
+      <c r="F79" s="10" t="inlineStr">
         <is>
           <t>마스터에 약관 KCD 목록이 있으면 대조 (없으면 조건 없이 계산하고 로그)</t>
         </is>
       </c>
-      <c r="G77" s="7" t="inlineStr">
+      <c r="G79" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H77" s="7" t="inlineStr">
+      <c r="H79" s="7" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I77" s="10" t="inlineStr">
+      <c r="I79" s="10" t="inlineStr">
         <is>
           <t>다빈치 로봇수술  (robot)</t>
         </is>
       </c>
-      <c r="J77" s="10" t="inlineStr"/>
-      <c r="K77" s="10" t="inlineStr"/>
-      <c r="L77" s="10" t="inlineStr"/>
-      <c r="M77" s="10" t="inlineStr">
+      <c r="J79" s="10" t="inlineStr"/>
+      <c r="K79" s="10" t="inlineStr"/>
+      <c r="L79" s="10" t="inlineStr"/>
+      <c r="M79" s="10" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N77" s="10" t="inlineStr">
+      <c r="N79" s="10" t="inlineStr">
         <is>
           <t>약관 대상 암(세부보장별 : 암(특정암제외) / 특정암 C61·C73)의 다빈치로봇 암수술 · 최초 1회</t>
         </is>
       </c>
-      <c r="O77" s="10" t="inlineStr">
+      <c r="O79" s="10" t="inlineStr">
         <is>
           <t>다빈치로봇 수술 치료비 — 설계서의 (특정암)·(암(특정암제외)) 표기는 마스터 세부보장 레코드로 매칭되어 그 KCD(codes_listed)로 판정 · 약관 제1조 「최초 1회에 한하여」(v8.61 : 종전 major_or_sim·연 1회로 특정암 줄이 모든 암에 붙었다)</t>
         </is>
       </c>
-      <c r="P77" s="7" t="n">
+      <c r="P79" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="Q77" s="10" t="inlineStr"/>
-      <c r="R77" s="10" t="inlineStr">
+      <c r="Q79" s="10" t="inlineStr"/>
+      <c r="R79" s="10" t="inlineStr">
         <is>
           <t>갱신형 다빈치로봇 암수술비
 갱신형 다빈치로봇 암수술비[암(특정암제외)]
@@ -6864,49 +7020,49 @@
 갱신형 다빈치로봇 암수술비(감액및면책기간미적용)[암(특정암제외)]</t>
         </is>
       </c>
-      <c r="S77" s="11" t="inlineStr"/>
-      <c r="T77" s="11" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="12" t="n">
-        <v>76</v>
-      </c>
-      <c r="B78" s="13" t="inlineStr">
+      <c r="S79" s="11" t="inlineStr"/>
+      <c r="T79" s="11" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
         <is>
           <t>tx_life_cancer</t>
         </is>
       </c>
-      <c r="C78" s="14" t="inlineStr">
+      <c r="C80" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D78" s="13" t="inlineStr">
+      <c r="D80" s="13" t="inlineStr">
         <is>
           <t>통합치료생활비|통합치료생활지원비</t>
         </is>
       </c>
-      <c r="E78" s="15" t="inlineStr">
+      <c r="E80" s="15" t="inlineStr">
         <is>
           <t>^유사암</t>
         </is>
       </c>
-      <c r="F78" s="15" t="inlineStr">
+      <c r="F80" s="15" t="inlineStr">
         <is>
           <t>암 — 유사암 제외 (약관 별표 암분류로 판정)</t>
         </is>
       </c>
-      <c r="G78" s="12" t="inlineStr">
+      <c r="G80" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H78" s="12" t="inlineStr">
+      <c r="H80" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I78" s="15" t="inlineStr">
+      <c r="I80" s="15" t="inlineStr">
         <is>
           <t>수술  (surg)
 항암 화학약물치료(급여)  (chemo)
@@ -6915,33 +7071,33 @@
 면역항암약물치료  (immune)</t>
         </is>
       </c>
-      <c r="J78" s="15" t="inlineStr"/>
-      <c r="K78" s="15" t="inlineStr"/>
-      <c r="L78" s="15" t="inlineStr">
+      <c r="J80" s="15" t="inlineStr"/>
+      <c r="K80" s="15" t="inlineStr"/>
+      <c r="L80" s="15" t="inlineStr">
         <is>
           <t>치료를 2회 이상 받은 단계에서만</t>
         </is>
       </c>
-      <c r="M78" s="15" t="inlineStr">
+      <c r="M80" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N78" s="15" t="inlineStr">
+      <c r="N80" s="15" t="inlineStr">
         <is>
           <t>연간 통합치료 2회 이상 · 연간 1회한</t>
         </is>
       </c>
-      <c r="O78" s="15" t="inlineStr">
+      <c r="O80" s="15" t="inlineStr">
         <is>
           <t>암(유사암제외) 통합치료 생활비 — 연간 통합치료(수술·항암약물·항암방사선) 2회 이상</t>
         </is>
       </c>
-      <c r="P78" s="12" t="n">
+      <c r="P80" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="Q78" s="15" t="inlineStr"/>
-      <c r="R78" s="15" t="inlineStr">
+      <c r="Q80" s="15" t="inlineStr"/>
+      <c r="R80" s="15" t="inlineStr">
         <is>
           <t>암 통합치료 생활비(연간 통합치료 2회이상)
 암(유사암제외) 통합치료 생활비(연간 통합치료 2회이상)
@@ -6950,155 +7106,155 @@
 특정순환계질환 통합치료 생활비[연간 통합치료 3회이상]</t>
         </is>
       </c>
-      <c r="S78" s="11" t="inlineStr"/>
-      <c r="T78" s="11" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="7" t="n">
-        <v>77</v>
-      </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="S80" s="11" t="inlineStr"/>
+      <c r="T80" s="11" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
         <is>
           <t>tx_life_sim</t>
         </is>
       </c>
-      <c r="C79" s="9" t="inlineStr">
+      <c r="C81" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D79" s="8" t="inlineStr">
+      <c r="D81" s="8" t="inlineStr">
         <is>
           <t>^유사암통합치료생활비</t>
         </is>
       </c>
-      <c r="E79" s="10" t="inlineStr"/>
-      <c r="F79" s="10" t="inlineStr">
+      <c r="E81" s="10" t="inlineStr"/>
+      <c r="F81" s="10" t="inlineStr">
         <is>
           <t>유사암 — 제자리암·경계성종양·갑상선암·기타피부암</t>
         </is>
       </c>
-      <c r="G79" s="7" t="inlineStr">
+      <c r="G81" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H79" s="7" t="inlineStr">
+      <c r="H81" s="7" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I79" s="10" t="inlineStr">
+      <c r="I81" s="10" t="inlineStr">
         <is>
           <t>수술  (surg)
 항암 화학약물치료(급여)  (chemo)
 항암 방사선치료  (rad)</t>
         </is>
       </c>
-      <c r="J79" s="10" t="inlineStr"/>
-      <c r="K79" s="10" t="inlineStr"/>
-      <c r="L79" s="10" t="inlineStr">
+      <c r="J81" s="10" t="inlineStr"/>
+      <c r="K81" s="10" t="inlineStr"/>
+      <c r="L81" s="10" t="inlineStr">
         <is>
           <t>치료를 2회 이상 받은 단계에서만</t>
         </is>
       </c>
-      <c r="M79" s="10" t="inlineStr">
+      <c r="M81" s="10" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N79" s="10" t="inlineStr">
+      <c r="N81" s="10" t="inlineStr">
         <is>
           <t>연간 유사암 통합치료 2회 이상 · 연간 1회한</t>
         </is>
       </c>
-      <c r="O79" s="10" t="inlineStr">
+      <c r="O81" s="10" t="inlineStr">
         <is>
           <t>유사암 통합치료 생활비</t>
         </is>
       </c>
-      <c r="P79" s="7" t="n">
+      <c r="P81" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="Q79" s="10" t="inlineStr"/>
-      <c r="R79" s="10" t="inlineStr">
+      <c r="Q81" s="10" t="inlineStr"/>
+      <c r="R81" s="10" t="inlineStr">
         <is>
           <t>유사암 통합치료 생활비(연간 통합치료 2회이상)
 유사암 통합치료 생활비(연간 통합치료 2회이상)</t>
         </is>
       </c>
-      <c r="S79" s="11" t="inlineStr"/>
-      <c r="T79" s="11" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="12" t="n">
-        <v>78</v>
-      </c>
-      <c r="B80" s="13" t="inlineStr">
+      <c r="S81" s="11" t="inlineStr"/>
+      <c r="T81" s="11" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
         <is>
           <t>tx_26</t>
         </is>
       </c>
-      <c r="C80" s="14" t="inlineStr">
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D80" s="13" t="inlineStr">
+      <c r="D82" s="13" t="inlineStr">
         <is>
           <t>26종항암방사선및약물치료비</t>
         </is>
       </c>
-      <c r="E80" s="15" t="inlineStr"/>
-      <c r="F80" s="15" t="inlineStr">
+      <c r="E82" s="15" t="inlineStr"/>
+      <c r="F82" s="15" t="inlineStr">
         <is>
           <t>암 — 유사암 제외 (약관 별표 암분류로 판정)</t>
         </is>
       </c>
-      <c r="G80" s="12" t="inlineStr">
+      <c r="G82" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H80" s="12" t="inlineStr">
+      <c r="H82" s="12" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I80" s="15" t="inlineStr">
+      <c r="I82" s="15" t="inlineStr">
         <is>
           <t>항암 화학약물치료(급여)  (chemo)
 항암 방사선치료  (rad)</t>
         </is>
       </c>
-      <c r="J80" s="15" t="inlineStr"/>
-      <c r="K80" s="15" t="inlineStr"/>
-      <c r="L80" s="15" t="inlineStr">
+      <c r="J82" s="15" t="inlineStr"/>
+      <c r="K82" s="15" t="inlineStr"/>
+      <c r="L82" s="15" t="inlineStr">
         <is>
           <t>세부급부 이름에서 치료행위·암종을 다시 읽음
 메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
         </is>
       </c>
-      <c r="M80" s="15" t="inlineStr">
+      <c r="M82" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N80" s="15" t="inlineStr">
+      <c r="N82" s="15" t="inlineStr">
         <is>
           <t>암종별 항암 치료 · 최초 1회</t>
         </is>
       </c>
-      <c r="O80" s="15" t="inlineStr">
+      <c r="O82" s="15" t="inlineStr">
         <is>
           <t>26종 항암방사선및약물치료비 — 세부급부 [항암방사선치료비(암종)]/[항암약물치료비(암종)]의 암종을 EMB.syn 코드로 판정</t>
         </is>
       </c>
-      <c r="P80" s="12" t="n">
+      <c r="P82" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="Q80" s="15" t="inlineStr"/>
-      <c r="R80" s="15" t="inlineStr">
+      <c r="Q82" s="15" t="inlineStr"/>
+      <c r="R82" s="15" t="inlineStr">
         <is>
           <t>26종 항암방사선및약물치료비 (전이포함)(유사암제외)
 26종 항암방사선및약물치료비 (전이포함)(유사암제외)(감액및면책기간미 적용)
@@ -7107,76 +7263,76 @@
 26종항암방사선및약물치료비(전이포함)(유사암제외)</t>
         </is>
       </c>
-      <c r="S80" s="11" t="inlineStr"/>
-      <c r="T80" s="11" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="S82" s="11" t="inlineStr"/>
+      <c r="T82" s="11" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
         <is>
           <t>tx_chemo</t>
         </is>
       </c>
-      <c r="C81" s="9" t="inlineStr">
+      <c r="C83" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D81" s="8" t="inlineStr">
+      <c r="D83" s="8" t="inlineStr">
         <is>
           <t>항암약물치료비</t>
         </is>
       </c>
-      <c r="E81" s="10" t="inlineStr">
+      <c r="E83" s="10" t="inlineStr">
         <is>
           <t>표적|면역|호르몬|방사선</t>
         </is>
       </c>
-      <c r="F81" s="10" t="inlineStr">
+      <c r="F83" s="10" t="inlineStr">
         <is>
           <t>암 또는 유사암</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr">
+      <c r="G83" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H81" s="7" t="inlineStr">
+      <c r="H83" s="7" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I81" s="10" t="inlineStr">
+      <c r="I83" s="10" t="inlineStr">
         <is>
           <t>항암 화학약물치료(급여)  (chemo)</t>
         </is>
       </c>
-      <c r="J81" s="10" t="inlineStr"/>
-      <c r="K81" s="10" t="inlineStr"/>
-      <c r="L81" s="10" t="inlineStr"/>
-      <c r="M81" s="10" t="inlineStr">
+      <c r="J83" s="10" t="inlineStr"/>
+      <c r="K83" s="10" t="inlineStr"/>
+      <c r="L83" s="10" t="inlineStr"/>
+      <c r="M83" s="10" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N81" s="10" t="inlineStr">
+      <c r="N83" s="10" t="inlineStr">
         <is>
           <t>항암약물치료 최초 1회</t>
         </is>
       </c>
-      <c r="O81" s="10" t="inlineStr">
+      <c r="O83" s="10" t="inlineStr">
         <is>
           <t>항암약물치료비(급여 항암약물치료)</t>
         </is>
       </c>
-      <c r="P81" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q81" s="10" t="inlineStr"/>
-      <c r="R81" s="10" t="inlineStr">
+      <c r="P83" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q83" s="10" t="inlineStr"/>
+      <c r="R83" s="10" t="inlineStr">
         <is>
           <t>비급여 항암약물치료비(전액본인부담 포함, 연간1회한, 10년간)
 암진단및치료비Ⅱ[항암약물치료비]
@@ -7185,73 +7341,73 @@
 암치료,후유장해및진단비[항암약물치료비]</t>
         </is>
       </c>
-      <c r="S81" s="11" t="inlineStr"/>
-      <c r="T81" s="11" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="B82" s="13" t="inlineStr">
+      <c r="S83" s="11" t="inlineStr"/>
+      <c r="T83" s="11" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" s="13" t="inlineStr">
         <is>
           <t>tx_chemo_rad</t>
         </is>
       </c>
-      <c r="C82" s="14" t="inlineStr">
+      <c r="C84" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D82" s="13" t="inlineStr">
+      <c r="D84" s="13" t="inlineStr">
         <is>
           <t>항암방사선(및)?약물치료비|26종항암방사선및약물치료비</t>
         </is>
       </c>
-      <c r="E82" s="15" t="inlineStr"/>
-      <c r="F82" s="15" t="inlineStr">
+      <c r="E84" s="15" t="inlineStr"/>
+      <c r="F84" s="15" t="inlineStr">
         <is>
           <t>암 또는 유사암</t>
         </is>
       </c>
-      <c r="G82" s="12" t="inlineStr">
+      <c r="G84" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H82" s="12" t="inlineStr">
+      <c r="H84" s="12" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I82" s="15" t="inlineStr">
+      <c r="I84" s="15" t="inlineStr">
         <is>
           <t>항암 화학약물치료(급여)  (chemo)
 항암 방사선치료  (rad)</t>
         </is>
       </c>
-      <c r="J82" s="15" t="inlineStr"/>
-      <c r="K82" s="15" t="inlineStr"/>
-      <c r="L82" s="15" t="inlineStr"/>
-      <c r="M82" s="15" t="inlineStr">
+      <c r="J84" s="15" t="inlineStr"/>
+      <c r="K84" s="15" t="inlineStr"/>
+      <c r="L84" s="15" t="inlineStr"/>
+      <c r="M84" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N82" s="15" t="inlineStr">
+      <c r="N84" s="15" t="inlineStr">
         <is>
           <t>항암방사선·약물치료 · 최초 1회</t>
         </is>
       </c>
-      <c r="O82" s="15" t="inlineStr">
+      <c r="O84" s="15" t="inlineStr">
         <is>
           <t>항암방사선·약물치료비</t>
         </is>
       </c>
-      <c r="P82" s="12" t="n">
+      <c r="P84" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="Q82" s="15" t="inlineStr"/>
-      <c r="R82" s="15" t="inlineStr">
+      <c r="Q84" s="15" t="inlineStr"/>
+      <c r="R84" s="15" t="inlineStr">
         <is>
           <t>항암방사선약물치료비
 계속받는 항암방사선약물치료비(급여)(연간1회한)
@@ -7260,142 +7416,142 @@
 계속받는 항암방사선약물치료비(급여)(연간1회한) (감액및면책기간미적용)</t>
         </is>
       </c>
-      <c r="S82" s="11" t="inlineStr"/>
-      <c r="T82" s="11" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="7" t="n">
-        <v>81</v>
-      </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="S84" s="11" t="inlineStr"/>
+      <c r="T84" s="11" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
         <is>
           <t>skip_recur_monthly</t>
         </is>
       </c>
-      <c r="C83" s="9" t="inlineStr">
+      <c r="C85" s="9" t="inlineStr">
         <is>
           <t>계산 제외 (제도성·조건부)</t>
         </is>
       </c>
-      <c r="D83" s="8" t="inlineStr">
+      <c r="D85" s="8" t="inlineStr">
         <is>
           <t>매월계속암치료비</t>
         </is>
       </c>
-      <c r="E83" s="10" t="inlineStr"/>
-      <c r="F83" s="10" t="inlineStr">
+      <c r="E85" s="10" t="inlineStr"/>
+      <c r="F85" s="10" t="inlineStr">
         <is>
           <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
         </is>
       </c>
-      <c r="G83" s="7" t="inlineStr">
+      <c r="G85" s="7" t="inlineStr">
         <is>
           <t>분류만 (금액 계산 안 함)</t>
         </is>
       </c>
-      <c r="H83" s="7" t="inlineStr">
+      <c r="H85" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I83" s="10" t="inlineStr"/>
-      <c r="J83" s="10" t="inlineStr"/>
-      <c r="K83" s="10" t="inlineStr"/>
-      <c r="L83" s="10" t="inlineStr">
+      <c r="I85" s="10" t="inlineStr"/>
+      <c r="J85" s="10" t="inlineStr"/>
+      <c r="K85" s="10" t="inlineStr"/>
+      <c r="L85" s="10" t="inlineStr">
         <is>
           <t>기록 사유 : 첫번째암 진단확정일부터 1년이 지난 뒤 계속암(기타피부암·갑상선암·전립선암 제외)으로 진단확정되면 가입금액을 매월 12회 지급하는 진단형 담보(통61 제1조) — 치료 행위와 무관하고 재진단 시점 조건이 있어 사례로 단정할 수 없어 계산 제외(v8.63)</t>
         </is>
       </c>
-      <c r="M83" s="10" t="inlineStr"/>
-      <c r="N83" s="10" t="inlineStr"/>
-      <c r="O83" s="10" t="inlineStr">
+      <c r="M85" s="10" t="inlineStr"/>
+      <c r="N85" s="10" t="inlineStr"/>
+      <c r="O85" s="10" t="inlineStr">
         <is>
           <t>매월 계속암치료비 — 1년 뒤 계속암 진단 조건부(사례 계산 제외)(v8.63)</t>
         </is>
       </c>
-      <c r="P83" s="7" t="n">
+      <c r="P85" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="Q83" s="10" t="inlineStr"/>
-      <c r="R83" s="10" t="inlineStr">
+      <c r="Q85" s="10" t="inlineStr"/>
+      <c r="R85" s="10" t="inlineStr">
         <is>
           <t>매월 계속암치료비
 매월계속암치료비
 매월계속암치료비</t>
         </is>
       </c>
-      <c r="S83" s="11" t="inlineStr"/>
-      <c r="T83" s="11" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="12" t="n">
-        <v>82</v>
-      </c>
-      <c r="B84" s="13" t="inlineStr">
+      <c r="S85" s="11" t="inlineStr"/>
+      <c r="T85" s="11" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" s="13" t="inlineStr">
         <is>
           <t>tx_cancer_main_sub</t>
         </is>
       </c>
-      <c r="C84" s="14" t="inlineStr">
+      <c r="C86" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D84" s="13" t="inlineStr">
+      <c r="D86" s="13" t="inlineStr">
         <is>
           <t>(특정소액암|특정소화기암|15대특정암|14대특정암|10대특정암|4대고액암|기타피부암및갑상선암)주요치료비</t>
         </is>
       </c>
-      <c r="E84" s="15" t="inlineStr"/>
-      <c r="F84" s="15" t="inlineStr">
+      <c r="E86" s="15" t="inlineStr"/>
+      <c r="F86" s="15" t="inlineStr">
         <is>
           <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
         </is>
       </c>
-      <c r="G84" s="12" t="inlineStr">
+      <c r="G86" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H84" s="12" t="inlineStr">
+      <c r="H86" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I84" s="15" t="inlineStr">
+      <c r="I86" s="15" t="inlineStr">
         <is>
           <t>수술  (surg)
 항암 화학약물치료(급여)  (chemo)
 항암 방사선치료  (rad)</t>
         </is>
       </c>
-      <c r="J84" s="15" t="inlineStr"/>
-      <c r="K84" s="15" t="inlineStr"/>
-      <c r="L84" s="15" t="inlineStr">
+      <c r="J86" s="15" t="inlineStr"/>
+      <c r="K86" s="15" t="inlineStr"/>
+      <c r="L86" s="15" t="inlineStr">
         <is>
           <t>메모 : 통합암 주요치료비의 암구분별 세부보장(통51-1~6·통52-1~6 등) — 세부보장 마스터 KCD 목록(특정소액암 10코드 등)으로 판정. 전에는 tx_cancer_main(암 전체)에 걸려 위암 수술에 특정소액암 주요치료비가 붙었다(v8.63)</t>
         </is>
       </c>
-      <c r="M84" s="15" t="inlineStr">
+      <c r="M86" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N84" s="15" t="inlineStr">
+      <c r="N86" s="15" t="inlineStr">
         <is>
           <t>약관 별표 통합암 분류표의 해당 암구분 진단 후 주요치료(수술·항암약물·항암방사선) · 연간 1회</t>
         </is>
       </c>
-      <c r="O84" s="15" t="inlineStr">
+      <c r="O86" s="15" t="inlineStr">
         <is>
           <t>통합암 주요치료비 암구분별 세부보장 — 세부보장 KCD 목록으로 판정(v8.63)</t>
         </is>
       </c>
-      <c r="P84" s="12" t="n">
+      <c r="P86" s="12" t="n">
         <v>64</v>
       </c>
-      <c r="Q84" s="15" t="inlineStr"/>
-      <c r="R84" s="15" t="inlineStr">
+      <c r="Q86" s="15" t="inlineStr"/>
+      <c r="R86" s="15" t="inlineStr">
         <is>
           <t>특정소액암 주요치료비(연간1회한, 10년간)
 특정소화기암 주요치료비(연간1회한, 10년간)
@@ -7404,74 +7560,78 @@
 4대고액암 주요치료비(연간1회한, 10년간)</t>
         </is>
       </c>
-      <c r="S84" s="11" t="inlineStr"/>
-      <c r="T84" s="11" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="7" t="n">
-        <v>83</v>
-      </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="S86" s="11" t="inlineStr"/>
+      <c r="T86" s="11" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
         <is>
           <t>tx_cancer_main</t>
         </is>
       </c>
-      <c r="C85" s="9" t="inlineStr">
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D85" s="8" t="inlineStr">
+      <c r="D87" s="8" t="inlineStr">
         <is>
           <t>암(\(유사암제외\))?주요치료비</t>
         </is>
       </c>
-      <c r="E85" s="10" t="inlineStr"/>
-      <c r="F85" s="10" t="inlineStr">
-        <is>
-          <t>암 또는 유사암</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="inlineStr">
+      <c r="E87" s="10" t="inlineStr"/>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>major_thy_skin</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H85" s="7" t="inlineStr">
+      <c r="H87" s="7" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I85" s="10" t="inlineStr">
+      <c r="I87" s="10" t="inlineStr">
         <is>
           <t>수술  (surg)
 항암 화학약물치료(급여)  (chemo)
 항암 방사선치료  (rad)</t>
         </is>
       </c>
-      <c r="J85" s="10" t="inlineStr"/>
-      <c r="K85" s="10" t="inlineStr"/>
-      <c r="L85" s="10" t="inlineStr"/>
-      <c r="M85" s="10" t="inlineStr">
+      <c r="J87" s="10" t="inlineStr"/>
+      <c r="K87" s="10" t="inlineStr"/>
+      <c r="L87" s="10" t="inlineStr">
+        <is>
+          <t>메모 : 통81·또125 제5조 암주요치료 = 암(유사암제외)·기타피부암·갑상선암의 치료(제자리암·경계성종양 아님)(v8.63)</t>
+        </is>
+      </c>
+      <c r="M87" s="10" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N85" s="10" t="inlineStr">
+      <c r="N87" s="10" t="inlineStr">
         <is>
           <t>암 주요치료(수술·항암·방사선) · 연간 1회</t>
         </is>
       </c>
-      <c r="O85" s="10" t="inlineStr">
+      <c r="O87" s="10" t="inlineStr">
         <is>
           <t>암 주요치료비</t>
         </is>
       </c>
-      <c r="P85" s="7" t="n">
+      <c r="P87" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="Q85" s="10" t="inlineStr"/>
-      <c r="R85" s="10" t="inlineStr">
+      <c r="Q87" s="10" t="inlineStr"/>
+      <c r="R87" s="10" t="inlineStr">
         <is>
           <t>암 주요치료비(연간1회한, 10년간)
 암(유사암제외) 주요치료비(연간1회한, 10년간)
@@ -7480,45 +7640,45 @@
 상급종합병원,국립암센터 암 주요치료비(연간1회한, 10년간)</t>
         </is>
       </c>
-      <c r="S85" s="11" t="inlineStr"/>
-      <c r="T85" s="11" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="12" t="n">
-        <v>84</v>
-      </c>
-      <c r="B86" s="13" t="inlineStr">
+      <c r="S87" s="11" t="inlineStr"/>
+      <c r="T87" s="11" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" s="13" t="inlineStr">
         <is>
           <t>tx_cancer_exam</t>
         </is>
       </c>
-      <c r="C86" s="14" t="inlineStr">
+      <c r="C88" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D86" s="13" t="inlineStr">
+      <c r="D88" s="13" t="inlineStr">
         <is>
           <t>암(CT촬영|MRI촬영|내시경|양전자단층촬영|초음파|특정단일유전자|특정생검|특정NGS).*검사비</t>
         </is>
       </c>
-      <c r="E86" s="15" t="inlineStr"/>
-      <c r="F86" s="15" t="inlineStr">
+      <c r="E88" s="15" t="inlineStr"/>
+      <c r="F88" s="15" t="inlineStr">
         <is>
           <t>암 또는 유사암</t>
         </is>
       </c>
-      <c r="G86" s="12" t="inlineStr">
+      <c r="G88" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H86" s="12" t="inlineStr">
+      <c r="H88" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I86" s="15" t="inlineStr">
+      <c r="I88" s="15" t="inlineStr">
         <is>
           <t>CT 검사  (x_ct)
 MRI 검사  (x_mri)
@@ -7530,33 +7690,33 @@
 NGS 유전자패널검사  (x_ngs)</t>
         </is>
       </c>
-      <c r="J86" s="15" t="inlineStr"/>
-      <c r="K86" s="15" t="inlineStr"/>
-      <c r="L86" s="15" t="inlineStr">
+      <c r="J88" s="15" t="inlineStr"/>
+      <c r="K88" s="15" t="inlineStr"/>
+      <c r="L88" s="15" t="inlineStr">
         <is>
           <t>약관이 진료행위(수가)코드를 열거한 항목은 그 목록에 있을 때만</t>
         </is>
       </c>
-      <c r="M86" s="15" t="inlineStr">
+      <c r="M88" s="15" t="inlineStr">
         <is>
           <t>암 치료</t>
         </is>
       </c>
-      <c r="N86" s="15" t="inlineStr">
+      <c r="N88" s="15" t="inlineStr">
         <is>
           <t>암 검사 · 연간 1회</t>
         </is>
       </c>
-      <c r="O86" s="15" t="inlineStr">
+      <c r="O88" s="15" t="inlineStr">
         <is>
           <t>암 검사비 — 약관이 진료행위(수가)코드를 열거한 항목(특정생검조직병리·특정단일유전자)은 마스터 수가코드 목록과 대조해 목록에 있을 때만 지급한다. 내시경·MRI·CT·PET·초음파는 약관이 분류번호 구간 전체를 대상으로 하므로 치료행위 키로 판정(v8.53)</t>
         </is>
       </c>
-      <c r="P86" s="12" t="n">
+      <c r="P88" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="Q86" s="15" t="inlineStr"/>
-      <c r="R86" s="15" t="inlineStr">
+      <c r="Q88" s="15" t="inlineStr"/>
+      <c r="R88" s="15" t="inlineStr">
         <is>
           <t>갱신형 암 MRI촬영검사비 (급여, 연간1회한)
 갱신형 암 양전자단층촬영(PET)검사비 (급여, 연간1회한)
@@ -7565,148 +7725,6 @@
 갱신형 암 CT촬영검사비 (급여,연간1회한)</t>
         </is>
       </c>
-      <c r="S86" s="11" t="inlineStr"/>
-      <c r="T86" s="11" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="7" t="n">
-        <v>85</v>
-      </c>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t>tx_cancer_rehab</t>
-        </is>
-      </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>치료비 (치료행위)</t>
-        </is>
-      </c>
-      <c r="D87" s="8" t="inlineStr">
-        <is>
-          <t>암특정재활치료비</t>
-        </is>
-      </c>
-      <c r="E87" s="10" t="inlineStr"/>
-      <c r="F87" s="10" t="inlineStr">
-        <is>
-          <t>major_thy_skin</t>
-        </is>
-      </c>
-      <c r="G87" s="7" t="inlineStr">
-        <is>
-          <t>계산함</t>
-        </is>
-      </c>
-      <c r="H87" s="7" t="inlineStr">
-        <is>
-          <t>연 1회</t>
-        </is>
-      </c>
-      <c r="I87" s="10" t="inlineStr">
-        <is>
-          <t>재활치료  (rehab)</t>
-        </is>
-      </c>
-      <c r="J87" s="10" t="inlineStr"/>
-      <c r="K87" s="10" t="inlineStr"/>
-      <c r="L87" s="10" t="inlineStr"/>
-      <c r="M87" s="10" t="inlineStr">
-        <is>
-          <t>암 치료</t>
-        </is>
-      </c>
-      <c r="N87" s="10" t="inlineStr">
-        <is>
-          <t>암 재활치료</t>
-        </is>
-      </c>
-      <c r="O87" s="10" t="inlineStr">
-        <is>
-          <t>암 재활치료비</t>
-        </is>
-      </c>
-      <c r="P87" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q87" s="10" t="inlineStr"/>
-      <c r="R87" s="10" t="inlineStr">
-        <is>
-          <t>암특정재활치료비(급여, 1일1회한, 연간20회한)
-암특정재활치료비(급여,1일1회한,연간20회한)</t>
-        </is>
-      </c>
-      <c r="S87" s="11" t="inlineStr"/>
-      <c r="T87" s="11" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="12" t="n">
-        <v>86</v>
-      </c>
-      <c r="B88" s="13" t="inlineStr">
-        <is>
-          <t>tx_cancer_pain</t>
-        </is>
-      </c>
-      <c r="C88" s="14" t="inlineStr">
-        <is>
-          <t>치료비 (치료행위)</t>
-        </is>
-      </c>
-      <c r="D88" s="13" t="inlineStr">
-        <is>
-          <t>암특정통증완화치료비</t>
-        </is>
-      </c>
-      <c r="E88" s="15" t="inlineStr"/>
-      <c r="F88" s="15" t="inlineStr">
-        <is>
-          <t>암 또는 유사암</t>
-        </is>
-      </c>
-      <c r="G88" s="12" t="inlineStr">
-        <is>
-          <t>계산함</t>
-        </is>
-      </c>
-      <c r="H88" s="12" t="inlineStr">
-        <is>
-          <t>연 1회</t>
-        </is>
-      </c>
-      <c r="I88" s="15" t="inlineStr">
-        <is>
-          <t>통증치료(신경차단 등)  (pain)</t>
-        </is>
-      </c>
-      <c r="J88" s="15" t="inlineStr"/>
-      <c r="K88" s="15" t="inlineStr"/>
-      <c r="L88" s="15" t="inlineStr"/>
-      <c r="M88" s="15" t="inlineStr">
-        <is>
-          <t>암 치료</t>
-        </is>
-      </c>
-      <c r="N88" s="15" t="inlineStr">
-        <is>
-          <t>통증완화치료 · 연간 1회</t>
-        </is>
-      </c>
-      <c r="O88" s="15" t="inlineStr">
-        <is>
-          <t>암 통증완화치료비</t>
-        </is>
-      </c>
-      <c r="P88" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q88" s="15" t="inlineStr"/>
-      <c r="R88" s="15" t="inlineStr">
-        <is>
-          <t>암특정통증완화치료비(급여, 연간1회한)
-암특정통증완화치료비(급여,연간1회한)</t>
-        </is>
-      </c>
       <c r="S88" s="11" t="inlineStr"/>
       <c r="T88" s="11" t="inlineStr"/>
     </row>
@@ -7716,7 +7734,7 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>tx_thromb</t>
+          <t>tx_cancer_rehab</t>
         </is>
       </c>
       <c r="C89" s="9" t="inlineStr">
@@ -7726,13 +7744,13 @@
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>혈전용해치료비</t>
+          <t>암특정재활치료비</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr"/>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
+          <t>major_thy_skin</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -7742,41 +7760,183 @@
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>최초 1회</t>
+          <t>연 1회</t>
         </is>
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>혈전용해치료(약물)  (thromb)</t>
+          <t>재활치료  (rehab)</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr"/>
       <c r="K89" s="10" t="inlineStr"/>
-      <c r="L89" s="10" t="inlineStr">
-        <is>
-          <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
-        </is>
-      </c>
+      <c r="L89" s="10" t="inlineStr"/>
       <c r="M89" s="10" t="inlineStr">
         <is>
-          <t>치료비</t>
+          <t>암 치료</t>
         </is>
       </c>
       <c r="N89" s="10" t="inlineStr">
         <is>
-          <t>혈전용해치료 · 최초 1회</t>
+          <t>암 재활치료</t>
         </is>
       </c>
       <c r="O89" s="10" t="inlineStr">
         <is>
-          <t>혈전용해치료비</t>
+          <t>암 재활치료비</t>
         </is>
       </c>
       <c r="P89" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Q89" s="10" t="inlineStr"/>
       <c r="R89" s="10" t="inlineStr">
+        <is>
+          <t>암특정재활치료비(급여, 1일1회한, 연간20회한)
+암특정재활치료비(급여,1일1회한,연간20회한)</t>
+        </is>
+      </c>
+      <c r="S89" s="11" t="inlineStr"/>
+      <c r="T89" s="11" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>tx_cancer_pain</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D90" s="13" t="inlineStr">
+        <is>
+          <t>암특정통증완화치료비</t>
+        </is>
+      </c>
+      <c r="E90" s="15" t="inlineStr"/>
+      <c r="F90" s="15" t="inlineStr">
+        <is>
+          <t>암 또는 유사암</t>
+        </is>
+      </c>
+      <c r="G90" s="12" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H90" s="12" t="inlineStr">
+        <is>
+          <t>연 1회</t>
+        </is>
+      </c>
+      <c r="I90" s="15" t="inlineStr">
+        <is>
+          <t>통증치료(신경차단 등)  (pain)</t>
+        </is>
+      </c>
+      <c r="J90" s="15" t="inlineStr"/>
+      <c r="K90" s="15" t="inlineStr"/>
+      <c r="L90" s="15" t="inlineStr"/>
+      <c r="M90" s="15" t="inlineStr">
+        <is>
+          <t>암 치료</t>
+        </is>
+      </c>
+      <c r="N90" s="15" t="inlineStr">
+        <is>
+          <t>통증완화치료 · 연간 1회</t>
+        </is>
+      </c>
+      <c r="O90" s="15" t="inlineStr">
+        <is>
+          <t>암 통증완화치료비</t>
+        </is>
+      </c>
+      <c r="P90" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q90" s="15" t="inlineStr"/>
+      <c r="R90" s="15" t="inlineStr">
+        <is>
+          <t>암특정통증완화치료비(급여, 연간1회한)
+암특정통증완화치료비(급여,연간1회한)</t>
+        </is>
+      </c>
+      <c r="S90" s="11" t="inlineStr"/>
+      <c r="T90" s="11" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>tx_thromb</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>혈전용해치료비</t>
+        </is>
+      </c>
+      <c r="E91" s="10" t="inlineStr"/>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>최초 1회</t>
+        </is>
+      </c>
+      <c r="I91" s="10" t="inlineStr">
+        <is>
+          <t>혈전용해치료(약물)  (thromb)</t>
+        </is>
+      </c>
+      <c r="J91" s="10" t="inlineStr"/>
+      <c r="K91" s="10" t="inlineStr"/>
+      <c r="L91" s="10" t="inlineStr">
+        <is>
+          <t>메모 : 약관 제1조 「최초 1회에 한하여」 — 담보명에 연간1회한·계속받는 이 있으면 연 1회(엔진 토큰). 전에는 연 1회로 계산해 GA 「반복(연 1회)」 칸에 매년 반복되는 것으로 보였다 (v8.63)</t>
+        </is>
+      </c>
+      <c r="M91" s="10" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N91" s="10" t="inlineStr">
+        <is>
+          <t>혈전용해치료 · 최초 1회</t>
+        </is>
+      </c>
+      <c r="O91" s="10" t="inlineStr">
+        <is>
+          <t>혈전용해치료비</t>
+        </is>
+      </c>
+      <c r="P91" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q91" s="10" t="inlineStr"/>
+      <c r="R91" s="10" t="inlineStr">
         <is>
           <t>혈전용해치료비Ⅱ
 혈전용해치료비Ⅱ(연간1회한)
@@ -7785,72 +7945,72 @@
 혈전용해치료비Ⅱ(연간1회한)</t>
         </is>
       </c>
-      <c r="S89" s="11" t="inlineStr"/>
-      <c r="T89" s="11" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="12" t="n">
-        <v>88</v>
-      </c>
-      <c r="B90" s="13" t="inlineStr">
+      <c r="S91" s="11" t="inlineStr"/>
+      <c r="T91" s="11" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" s="13" t="inlineStr">
         <is>
           <t>tx_thrombectomy</t>
         </is>
       </c>
-      <c r="C90" s="14" t="inlineStr">
+      <c r="C92" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D90" s="13" t="inlineStr">
+      <c r="D92" s="13" t="inlineStr">
         <is>
           <t>기계적혈전제거술.*치료비</t>
         </is>
       </c>
-      <c r="E90" s="15" t="inlineStr"/>
-      <c r="F90" s="15" t="inlineStr">
+      <c r="E92" s="15" t="inlineStr"/>
+      <c r="F92" s="15" t="inlineStr">
         <is>
           <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
         </is>
       </c>
-      <c r="G90" s="12" t="inlineStr">
+      <c r="G92" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H90" s="12" t="inlineStr">
+      <c r="H92" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I90" s="15" t="inlineStr">
+      <c r="I92" s="15" t="inlineStr">
         <is>
           <t>기계적 혈전제거술  (thrombectomy)</t>
         </is>
       </c>
-      <c r="J90" s="15" t="inlineStr"/>
-      <c r="K90" s="15" t="inlineStr"/>
-      <c r="L90" s="15" t="inlineStr"/>
-      <c r="M90" s="15" t="inlineStr">
+      <c r="J92" s="15" t="inlineStr"/>
+      <c r="K92" s="15" t="inlineStr"/>
+      <c r="L92" s="15" t="inlineStr"/>
+      <c r="M92" s="15" t="inlineStr">
         <is>
           <t>치료비</t>
         </is>
       </c>
-      <c r="N90" s="15" t="inlineStr">
+      <c r="N92" s="15" t="inlineStr">
         <is>
           <t>기계적 혈전제거술 · 연간 1회</t>
         </is>
       </c>
-      <c r="O90" s="15" t="inlineStr">
+      <c r="O92" s="15" t="inlineStr">
         <is>
           <t>기계적혈전제거술 치료비</t>
         </is>
       </c>
-      <c r="P90" s="12" t="n">
+      <c r="P92" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="Q90" s="15" t="inlineStr"/>
-      <c r="R90" s="15" t="inlineStr">
+      <c r="Q92" s="15" t="inlineStr"/>
+      <c r="R92" s="15" t="inlineStr">
         <is>
           <t>기계적혈전제거술(카테터법)치료비Ⅱ (급여, 연간1회한)
 기계적혈전제거술(카테터법)치료비Ⅱ(뇌졸중)(급여, 연간1회한)
@@ -7859,64 +8019,64 @@
 기계적혈전제거술(카테터법)치료비Ⅱ(뇌졸중)(급여, 연간1회한)(감액기간미적용)</t>
         </is>
       </c>
-      <c r="S90" s="11" t="inlineStr"/>
-      <c r="T90" s="11" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="7" t="n">
-        <v>89</v>
-      </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="S92" s="11" t="inlineStr"/>
+      <c r="T92" s="11" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
         <is>
           <t>skip_point_type</t>
         </is>
       </c>
-      <c r="C91" s="9" t="inlineStr">
+      <c r="C93" s="9" t="inlineStr">
         <is>
           <t>계산 제외 (제도성·조건부)</t>
         </is>
       </c>
-      <c r="D91" s="8" t="inlineStr">
+      <c r="D93" s="8" t="inlineStr">
         <is>
           <t>최대두배받는2대질환치료비</t>
         </is>
       </c>
-      <c r="E91" s="10" t="inlineStr"/>
-      <c r="F91" s="10" t="inlineStr">
+      <c r="E93" s="10" t="inlineStr"/>
+      <c r="F93" s="10" t="inlineStr">
         <is>
           <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
         </is>
       </c>
-      <c r="G91" s="7" t="inlineStr">
+      <c r="G93" s="7" t="inlineStr">
         <is>
           <t>분류만 (금액 계산 안 함)</t>
         </is>
       </c>
-      <c r="H91" s="7" t="inlineStr">
+      <c r="H93" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I91" s="10" t="inlineStr"/>
-      <c r="J91" s="10" t="inlineStr"/>
-      <c r="K91" s="10" t="inlineStr"/>
-      <c r="L91" s="10" t="inlineStr">
+      <c r="I93" s="10" t="inlineStr"/>
+      <c r="J93" s="10" t="inlineStr"/>
+      <c r="K93" s="10" t="inlineStr"/>
+      <c r="L93" s="10" t="inlineStr">
         <is>
           <t>기록 사유 : 포인트적립형 담보 — 치료마다 점수(비관혈수술·혈전용해 1점, 관혈수술 2점, 중환자실 4일 이상 1점·8일 이상 2점, 치료군별 최고점)를 쌓아 누적 1·2·3·4점 구간마다 가입금액의 25%·35%·40%·100%를 각각 최초 1회 지급(통106·케179 제2조·제5조) — 사례 한 단계로 점수를 정할 수 없어 계산 제외(v8.63)</t>
         </is>
       </c>
-      <c r="M91" s="10" t="inlineStr"/>
-      <c r="N91" s="10" t="inlineStr"/>
-      <c r="O91" s="10" t="inlineStr">
+      <c r="M93" s="10" t="inlineStr"/>
+      <c r="N93" s="10" t="inlineStr"/>
+      <c r="O93" s="10" t="inlineStr">
         <is>
           <t>최대두배받는2대질환치료비(포인트적립형) — 누적 점수 조건부(사례 계산 제외)(v8.63)</t>
         </is>
       </c>
-      <c r="P91" s="7" t="n">
+      <c r="P93" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="Q91" s="10" t="inlineStr"/>
-      <c r="R91" s="10" t="inlineStr">
+      <c r="Q93" s="10" t="inlineStr"/>
+      <c r="R93" s="10" t="inlineStr">
         <is>
           <t>최대두배받는2대질환치료비(포인트적립형)
 최대두배받는2대질환치료비(포인트적립형)[1점이상]
@@ -7925,73 +8085,73 @@
 최대두배받는2대질환치료비(포인트적립형)[4점이상]</t>
         </is>
       </c>
-      <c r="S91" s="11" t="inlineStr"/>
-      <c r="T91" s="11" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="B92" s="13" t="inlineStr">
+      <c r="S93" s="11" t="inlineStr"/>
+      <c r="T93" s="11" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" s="13" t="inlineStr">
         <is>
           <t>tx_two_major</t>
         </is>
       </c>
-      <c r="C92" s="14" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D92" s="13" t="inlineStr">
+      <c r="D94" s="13" t="inlineStr">
         <is>
           <t>2대질환.*(주요치료비|치료비)</t>
         </is>
       </c>
-      <c r="E92" s="15" t="inlineStr"/>
-      <c r="F92" s="15" t="inlineStr">
+      <c r="E94" s="15" t="inlineStr"/>
+      <c r="F94" s="15" t="inlineStr">
         <is>
           <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
         </is>
       </c>
-      <c r="G92" s="12" t="inlineStr">
+      <c r="G94" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H92" s="12" t="inlineStr">
+      <c r="H94" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I92" s="15" t="inlineStr">
+      <c r="I94" s="15" t="inlineStr">
         <is>
           <t>수술  (surg)
 혈전용해치료(약물)  (thromb)</t>
         </is>
       </c>
-      <c r="J92" s="15" t="inlineStr"/>
-      <c r="K92" s="15" t="inlineStr"/>
-      <c r="L92" s="15" t="inlineStr"/>
-      <c r="M92" s="15" t="inlineStr">
+      <c r="J94" s="15" t="inlineStr"/>
+      <c r="K94" s="15" t="inlineStr"/>
+      <c r="L94" s="15" t="inlineStr"/>
+      <c r="M94" s="15" t="inlineStr">
         <is>
           <t>치료비</t>
         </is>
       </c>
-      <c r="N92" s="15" t="inlineStr">
+      <c r="N94" s="15" t="inlineStr">
         <is>
           <t>뇌·심장 주요치료 · 연간 1회</t>
         </is>
       </c>
-      <c r="O92" s="15" t="inlineStr">
+      <c r="O94" s="15" t="inlineStr">
         <is>
           <t>2대질환 주요치료비</t>
         </is>
       </c>
-      <c r="P92" s="12" t="n">
+      <c r="P94" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="Q92" s="15" t="inlineStr"/>
-      <c r="R92" s="15" t="inlineStr">
+      <c r="Q94" s="15" t="inlineStr"/>
+      <c r="R94" s="15" t="inlineStr">
         <is>
           <t>2대질환 주요치료비(연간1회한, 10년간)
 상급종합병원 2대질환 주요치료비(연간1회한, 10년간)
@@ -8000,64 +8160,64 @@
 갱신형 2대질환 주요치료비(연간1회한, 10년간)</t>
         </is>
       </c>
-      <c r="S92" s="11" t="inlineStr"/>
-      <c r="T92" s="11" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="7" t="n">
-        <v>91</v>
-      </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="S94" s="11" t="inlineStr"/>
+      <c r="T94" s="11" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
         <is>
           <t>tx_dementia_target</t>
         </is>
       </c>
-      <c r="C93" s="9" t="inlineStr">
+      <c r="C95" s="9" t="inlineStr">
         <is>
           <t>계산 제외 (제도성·조건부)</t>
         </is>
       </c>
-      <c r="D93" s="8" t="inlineStr">
+      <c r="D95" s="8" t="inlineStr">
         <is>
           <t>표적치매약물허가치료비</t>
         </is>
       </c>
-      <c r="E93" s="10" t="inlineStr"/>
-      <c r="F93" s="10" t="inlineStr">
+      <c r="E95" s="10" t="inlineStr"/>
+      <c r="F95" s="10" t="inlineStr">
         <is>
           <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
         </is>
       </c>
-      <c r="G93" s="7" t="inlineStr">
+      <c r="G95" s="7" t="inlineStr">
         <is>
           <t>분류만 (금액 계산 안 함)</t>
         </is>
       </c>
-      <c r="H93" s="7" t="inlineStr">
+      <c r="H95" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I93" s="10" t="inlineStr"/>
-      <c r="J93" s="10" t="inlineStr"/>
-      <c r="K93" s="10" t="inlineStr"/>
-      <c r="L93" s="10" t="inlineStr">
+      <c r="I95" s="10" t="inlineStr"/>
+      <c r="J95" s="10" t="inlineStr"/>
+      <c r="K95" s="10" t="inlineStr"/>
+      <c r="L95" s="10" t="inlineStr">
         <is>
           <t>기록 사유 : 최경증 치매·경증 알츠하이머치매 진단 + 아밀로이드베타 적응증(PET 30 센틸로이드 이상 등) + 표적치매약물허가치료 N회 이상(7·13·19회)이 지급사유(제1조·제3조) — 사례로 단정할 수 없어 계산 제외</t>
         </is>
       </c>
-      <c r="M93" s="10" t="inlineStr"/>
-      <c r="N93" s="10" t="inlineStr"/>
-      <c r="O93" s="10" t="inlineStr">
+      <c r="M95" s="10" t="inlineStr"/>
+      <c r="N95" s="10" t="inlineStr"/>
+      <c r="O95" s="10" t="inlineStr">
         <is>
           <t>표적치매약물허가치료비(통265~268) — 치매 상태·검사·치료 횟수 조건부(사례 계산 제외). 종전 tx_etc_care 가 F00·G30 진단만으로 4단(기본·7회·13회·19회)을 한꺼번에 지급 계산(v8.61)</t>
         </is>
       </c>
-      <c r="P93" s="7" t="n">
+      <c r="P95" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="Q93" s="10" t="inlineStr"/>
-      <c r="R93" s="10" t="inlineStr">
+      <c r="Q95" s="10" t="inlineStr"/>
+      <c r="R95" s="10" t="inlineStr">
         <is>
           <t>갱신형 표적치매약물허가치료비 (최경증 치매,경증 알츠하이머치매)
 갱신형 표적치매약물허가치료비 (최경증 치매,경증 알츠하이머치매) (7회이상)
@@ -8066,192 +8226,67 @@
 갱신형 표적치매약물허가치료비 (최경증 치매,경증 알츠하이머치매)</t>
         </is>
       </c>
-      <c r="S93" s="11" t="inlineStr"/>
-      <c r="T93" s="11" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="12" t="n">
-        <v>92</v>
-      </c>
-      <c r="B94" s="13" t="inlineStr">
+      <c r="S95" s="11" t="inlineStr"/>
+      <c r="T95" s="11" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" s="13" t="inlineStr">
         <is>
           <t>tx_hyperthyroid</t>
         </is>
       </c>
-      <c r="C94" s="14" t="inlineStr">
+      <c r="C96" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D94" s="13" t="inlineStr">
+      <c r="D96" s="13" t="inlineStr">
         <is>
           <t>갑상선기능항진증치료비</t>
         </is>
       </c>
-      <c r="E94" s="15" t="inlineStr"/>
-      <c r="F94" s="15" t="inlineStr">
+      <c r="E96" s="15" t="inlineStr"/>
+      <c r="F96" s="15" t="inlineStr">
         <is>
           <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
         </is>
       </c>
-      <c r="G94" s="12" t="inlineStr">
+      <c r="G96" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H94" s="12" t="inlineStr">
+      <c r="H96" s="12" t="inlineStr">
         <is>
           <t>최초 1회</t>
         </is>
       </c>
-      <c r="I94" s="15" t="inlineStr">
+      <c r="I96" s="15" t="inlineStr">
         <is>
           <t>수술  (surg)
 ※ 이름 미정  (rai)
 ※ 이름 미정  (antithyroid60)</t>
         </is>
       </c>
-      <c r="J94" s="15" t="inlineStr"/>
-      <c r="K94" s="15" t="inlineStr"/>
-      <c r="L94" s="15" t="inlineStr"/>
-      <c r="M94" s="15" t="inlineStr">
-        <is>
-          <t>치료비</t>
-        </is>
-      </c>
-      <c r="N94" s="15" t="inlineStr">
-        <is>
-          <t>갑상선기능항진증 진단 후 갑상선절제술 · 방사성요오드치료 · 60일 이상 항갑상선제 처방 중 하나 · 최초 1회</t>
-        </is>
-      </c>
-      <c r="O94" s="15" t="inlineStr">
-        <is>
-          <t>갑상선기능항진증치료비(케87) — 제3조③의 세 치료(갑상선절제술 / 방사성요오드 / 항갑상선제 60일 이상 처방) 중 하나를 받아야 지급. 종전 tx_etc_care(치료행위 없음)가 E05 진단만으로 지급 계산(v8.61)</t>
-        </is>
-      </c>
-      <c r="P94" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q94" s="15" t="inlineStr"/>
-      <c r="R94" s="15" t="inlineStr">
-        <is>
-          <t>갑상선기능항진증치료비</t>
-        </is>
-      </c>
-      <c r="S94" s="11" t="inlineStr"/>
-      <c r="T94" s="11" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="7" t="n">
-        <v>93</v>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
-        <is>
-          <t>tx_cancer_adverse_drug</t>
-        </is>
-      </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>계산 제외 (제도성·조건부)</t>
-        </is>
-      </c>
-      <c r="D95" s="8" t="inlineStr">
-        <is>
-          <t>특정항암부작용약제치료비</t>
-        </is>
-      </c>
-      <c r="E95" s="10" t="inlineStr"/>
-      <c r="F95" s="10" t="inlineStr">
-        <is>
-          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
-        </is>
-      </c>
-      <c r="G95" s="7" t="inlineStr">
-        <is>
-          <t>분류만 (금액 계산 안 함)</t>
-        </is>
-      </c>
-      <c r="H95" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I95" s="10" t="inlineStr"/>
-      <c r="J95" s="10" t="inlineStr"/>
-      <c r="K95" s="10" t="inlineStr"/>
-      <c r="L95" s="10" t="inlineStr">
-        <is>
-          <t>기록 사유 : 암 진단 후 특정암합병증및항암부작용약제(급여) 또는 특정항구토제(급여)를 투약처방 받은 때 구분별(100% / 3%)로 지급(제1조·제4조) — 사례에 약제 처방 구분이 없어 계산 제외</t>
-        </is>
-      </c>
-      <c r="M95" s="10" t="inlineStr"/>
-      <c r="N95" s="10" t="inlineStr"/>
-      <c r="O95" s="10" t="inlineStr">
-        <is>
-          <t>특정항암부작용약제치료비(또124) — 약제 처방 조건부(사례 계산 제외). 종전 tx_etc_care 가 암 진단만으로 가입금액 전액을 지급 계산(v8.61)</t>
-        </is>
-      </c>
-      <c r="P95" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q95" s="10" t="inlineStr"/>
-      <c r="R95" s="10" t="inlineStr">
-        <is>
-          <t>특정항암부작용약제치료비(급여,연간1회한)
-특정항암부작용약제치료비(급여,연간1회한)</t>
-        </is>
-      </c>
-      <c r="S95" s="11" t="inlineStr"/>
-      <c r="T95" s="11" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="12" t="n">
-        <v>94</v>
-      </c>
-      <c r="B96" s="13" t="inlineStr">
-        <is>
-          <t>tx_arrhythmia_exam</t>
-        </is>
-      </c>
-      <c r="C96" s="14" t="inlineStr">
-        <is>
-          <t>계산 제외 (제도성·조건부)</t>
-        </is>
-      </c>
-      <c r="D96" s="13" t="inlineStr">
-        <is>
-          <t>부정맥질환특정검사비</t>
-        </is>
-      </c>
-      <c r="E96" s="15" t="inlineStr"/>
-      <c r="F96" s="15" t="inlineStr">
-        <is>
-          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
-        </is>
-      </c>
-      <c r="G96" s="12" t="inlineStr">
-        <is>
-          <t>분류만 (금액 계산 안 함)</t>
-        </is>
-      </c>
-      <c r="H96" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I96" s="15" t="inlineStr"/>
       <c r="J96" s="15" t="inlineStr"/>
       <c r="K96" s="15" t="inlineStr"/>
-      <c r="L96" s="15" t="inlineStr">
-        <is>
-          <t>기록 사유 : 부정맥질환 진단·치료 소견으로 별표(부정맥질환특정검사(급여) 분류표)의 검사(1종·2종)를 받은 때 지급(제2조·제5조) — 마스터에 수가코드 목록이 없고 사례에 검사 구분이 없어 계산 제외</t>
-        </is>
-      </c>
-      <c r="M96" s="15" t="inlineStr"/>
-      <c r="N96" s="15" t="inlineStr"/>
+      <c r="L96" s="15" t="inlineStr"/>
+      <c r="M96" s="15" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N96" s="15" t="inlineStr">
+        <is>
+          <t>갑상선기능항진증 진단 후 갑상선절제술 · 방사성요오드치료 · 60일 이상 항갑상선제 처방 중 하나 · 최초 1회</t>
+        </is>
+      </c>
       <c r="O96" s="15" t="inlineStr">
         <is>
-          <t>부정맥질환특정검사비(케345) — 별표 수가코드 검사 조건부(사례 계산 제외). 종전 tx_etc_care 가 I47·I48 진단만으로 지급 계산(v8.61)</t>
+          <t>갑상선기능항진증치료비(케87) — 제3조③의 세 치료(갑상선절제술 / 방사성요오드 / 항갑상선제 60일 이상 처방) 중 하나를 받아야 지급. 종전 tx_etc_care(치료행위 없음)가 E05 진단만으로 지급 계산(v8.61)</t>
         </is>
       </c>
       <c r="P96" s="12" t="n">
@@ -8260,7 +8295,7 @@
       <c r="Q96" s="15" t="inlineStr"/>
       <c r="R96" s="15" t="inlineStr">
         <is>
-          <t>갱신형 부정맥질환특정검사비</t>
+          <t>갑상선기능항진증치료비</t>
         </is>
       </c>
       <c r="S96" s="11" t="inlineStr"/>
@@ -8272,33 +8307,33 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>tx_hc_kcd</t>
+          <t>tx_cancer_adverse_drug</t>
         </is>
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>치료비 (치료행위)</t>
+          <t>계산 제외 (제도성·조건부)</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>(갑상선질환고주파열치료비|유방병변진공보조장치이용절제치료비|자궁근종고강도초음파집속술치료비)</t>
+          <t>특정항암부작용약제치료비</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr"/>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
+          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>계산함</t>
+          <t>분류만 (금액 계산 안 함)</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>최초 1회</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I97" s="10" t="inlineStr"/>
@@ -8306,29 +8341,154 @@
       <c r="K97" s="10" t="inlineStr"/>
       <c r="L97" s="10" t="inlineStr">
         <is>
-          <t>약관이 진료행위(수가)코드를 열거한 항목은 그 목록에 있을 때만</t>
-        </is>
-      </c>
-      <c r="M97" s="10" t="inlineStr">
-        <is>
-          <t>치료비</t>
-        </is>
-      </c>
-      <c r="N97" s="10" t="inlineStr">
-        <is>
-          <t>약관 대상 질병 진단 후 약관이 정한 시술(수가코드) · 최초 1회</t>
-        </is>
-      </c>
+          <t>기록 사유 : 암 진단 후 특정암합병증및항암부작용약제(급여) 또는 특정항구토제(급여)를 투약처방 받은 때 구분별(100% / 3%)로 지급(제1조·제4조) — 사례에 약제 처방 구분이 없어 계산 제외</t>
+        </is>
+      </c>
+      <c r="M97" s="10" t="inlineStr"/>
+      <c r="N97" s="10" t="inlineStr"/>
       <c r="O97" s="10" t="inlineStr">
         <is>
-          <t>갑상선 고주파열치료(PZ612) · 유방 진공보조절제(신의료기술 770) · 자궁근종 HIFU(RZ566) 치료비(케328) — 대상 질병(D34·E04 / D24·N60 / D25) + 그 시술의 수가코드가 사례에 있을 때만. 종전에는 갑상선 고주파열치료비가 tx_procedure(수술이면 지급)로, 나머지 둘은 tx_etc_care(진단만으로 지급)로 계산됐다(v8.61)</t>
+          <t>특정항암부작용약제치료비(또124) — 약제 처방 조건부(사례 계산 제외). 종전 tx_etc_care 가 암 진단만으로 가입금액 전액을 지급 계산(v8.61)</t>
         </is>
       </c>
       <c r="P97" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q97" s="10" t="inlineStr"/>
       <c r="R97" s="10" t="inlineStr">
+        <is>
+          <t>특정항암부작용약제치료비(급여,연간1회한)
+특정항암부작용약제치료비(급여,연간1회한)</t>
+        </is>
+      </c>
+      <c r="S97" s="11" t="inlineStr"/>
+      <c r="T97" s="11" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="12" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>tx_arrhythmia_exam</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>계산 제외 (제도성·조건부)</t>
+        </is>
+      </c>
+      <c r="D98" s="13" t="inlineStr">
+        <is>
+          <t>부정맥질환특정검사비</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr"/>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
+        </is>
+      </c>
+      <c r="G98" s="12" t="inlineStr">
+        <is>
+          <t>분류만 (금액 계산 안 함)</t>
+        </is>
+      </c>
+      <c r="H98" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I98" s="15" t="inlineStr"/>
+      <c r="J98" s="15" t="inlineStr"/>
+      <c r="K98" s="15" t="inlineStr"/>
+      <c r="L98" s="15" t="inlineStr">
+        <is>
+          <t>기록 사유 : 부정맥질환 진단·치료 소견으로 별표(부정맥질환특정검사(급여) 분류표)의 검사(1종·2종)를 받은 때 지급(제2조·제5조) — 마스터에 수가코드 목록이 없고 사례에 검사 구분이 없어 계산 제외</t>
+        </is>
+      </c>
+      <c r="M98" s="15" t="inlineStr"/>
+      <c r="N98" s="15" t="inlineStr"/>
+      <c r="O98" s="15" t="inlineStr">
+        <is>
+          <t>부정맥질환특정검사비(케345) — 별표 수가코드 검사 조건부(사례 계산 제외). 종전 tx_etc_care 가 I47·I48 진단만으로 지급 계산(v8.61)</t>
+        </is>
+      </c>
+      <c r="P98" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q98" s="15" t="inlineStr"/>
+      <c r="R98" s="15" t="inlineStr">
+        <is>
+          <t>갱신형 부정맥질환특정검사비</t>
+        </is>
+      </c>
+      <c r="S98" s="11" t="inlineStr"/>
+      <c r="T98" s="11" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="n">
+        <v>97</v>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>tx_hc_kcd</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>(갑상선질환고주파열치료비|유방병변진공보조장치이용절제치료비|자궁근종고강도초음파집속술치료비)</t>
+        </is>
+      </c>
+      <c r="E99" s="10" t="inlineStr"/>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
+          <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H99" s="7" t="inlineStr">
+        <is>
+          <t>최초 1회</t>
+        </is>
+      </c>
+      <c r="I99" s="10" t="inlineStr"/>
+      <c r="J99" s="10" t="inlineStr"/>
+      <c r="K99" s="10" t="inlineStr"/>
+      <c r="L99" s="10" t="inlineStr">
+        <is>
+          <t>약관이 진료행위(수가)코드를 열거한 항목은 그 목록에 있을 때만</t>
+        </is>
+      </c>
+      <c r="M99" s="10" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N99" s="10" t="inlineStr">
+        <is>
+          <t>약관 대상 질병 진단 후 약관이 정한 시술(수가코드) · 최초 1회</t>
+        </is>
+      </c>
+      <c r="O99" s="10" t="inlineStr">
+        <is>
+          <t>갑상선 고주파열치료(PZ612) · 유방 진공보조절제(신의료기술 770) · 자궁근종 HIFU(RZ566) 치료비(케328) — 대상 질병(D34·E04 / D24·N60 / D25) + 그 시술의 수가코드가 사례에 있을 때만. 종전에는 갑상선 고주파열치료비가 tx_procedure(수술이면 지급)로, 나머지 둘은 tx_etc_care(진단만으로 지급)로 계산됐다(v8.61)</t>
+        </is>
+      </c>
+      <c r="P99" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q99" s="10" t="inlineStr"/>
+      <c r="R99" s="10" t="inlineStr">
         <is>
           <t>갱신형 갑상선질환 고주파열치료비(최초1회한)
 갱신형 유방병변 진공보조장치이용절제치료비(최초1회한)
@@ -8337,148 +8497,6 @@
 갱신형특정질환3대치료비[갑상선질환 고주파열치료비(최초1회한)]</t>
         </is>
       </c>
-      <c r="S97" s="11" t="inlineStr"/>
-      <c r="T97" s="11" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="12" t="n">
-        <v>96</v>
-      </c>
-      <c r="B98" s="13" t="inlineStr">
-        <is>
-          <t>tx_anesth6</t>
-        </is>
-      </c>
-      <c r="C98" s="14" t="inlineStr">
-        <is>
-          <t>치료비 (치료행위)</t>
-        </is>
-      </c>
-      <c r="D98" s="13" t="inlineStr">
-        <is>
-          <t>전신마취치료비\(급여,6시간이상\)</t>
-        </is>
-      </c>
-      <c r="E98" s="15" t="inlineStr"/>
-      <c r="F98" s="15" t="inlineStr">
-        <is>
-          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
-        </is>
-      </c>
-      <c r="G98" s="12" t="inlineStr">
-        <is>
-          <t>계산함</t>
-        </is>
-      </c>
-      <c r="H98" s="12" t="inlineStr">
-        <is>
-          <t>받을 때마다</t>
-        </is>
-      </c>
-      <c r="I98" s="15" t="inlineStr">
-        <is>
-          <t>6시간 이상 전신마취 수술  (anes6)</t>
-        </is>
-      </c>
-      <c r="J98" s="15" t="inlineStr"/>
-      <c r="K98" s="15" t="inlineStr"/>
-      <c r="L98" s="15" t="inlineStr"/>
-      <c r="M98" s="15" t="inlineStr">
-        <is>
-          <t>치료비</t>
-        </is>
-      </c>
-      <c r="N98" s="15" t="inlineStr">
-        <is>
-          <t>종합병원 전신마취 6시간 이상 · 치료 1회당</t>
-        </is>
-      </c>
-      <c r="O98" s="15" t="inlineStr">
-        <is>
-          <t>종합병원 전신마취치료비(급여, 6시간이상) — 약관 제1조 '전신마취치료(급여)를 6시간 이상 받은 때 치료 1회당' · 제2조① 마취시간은 1회당 기준(합산 없음) · 연간 횟수 제한 없음(v8.61)</t>
-        </is>
-      </c>
-      <c r="P98" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q98" s="15" t="inlineStr"/>
-      <c r="R98" s="15" t="inlineStr">
-        <is>
-          <t>종합병원 전신마취치료비 (급여, 6시간이상)
-종합병원 전신마취치료비 (급여, 6시간이상)</t>
-        </is>
-      </c>
-      <c r="S98" s="11" t="inlineStr"/>
-      <c r="T98" s="11" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="7" t="n">
-        <v>97</v>
-      </c>
-      <c r="B99" s="8" t="inlineStr">
-        <is>
-          <t>tx_anesth4</t>
-        </is>
-      </c>
-      <c r="C99" s="9" t="inlineStr">
-        <is>
-          <t>치료비 (치료행위)</t>
-        </is>
-      </c>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>전신마취치료비\(급여,4시간이상\)</t>
-        </is>
-      </c>
-      <c r="E99" s="10" t="inlineStr"/>
-      <c r="F99" s="10" t="inlineStr">
-        <is>
-          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
-        </is>
-      </c>
-      <c r="G99" s="7" t="inlineStr">
-        <is>
-          <t>계산함</t>
-        </is>
-      </c>
-      <c r="H99" s="7" t="inlineStr">
-        <is>
-          <t>받을 때마다</t>
-        </is>
-      </c>
-      <c r="I99" s="10" t="inlineStr">
-        <is>
-          <t>4시간 이상 전신마취 수술  (anes4)</t>
-        </is>
-      </c>
-      <c r="J99" s="10" t="inlineStr"/>
-      <c r="K99" s="10" t="inlineStr"/>
-      <c r="L99" s="10" t="inlineStr"/>
-      <c r="M99" s="10" t="inlineStr">
-        <is>
-          <t>치료비</t>
-        </is>
-      </c>
-      <c r="N99" s="10" t="inlineStr">
-        <is>
-          <t>종합병원 전신마취 4시간 이상 · 치료 1회당</t>
-        </is>
-      </c>
-      <c r="O99" s="10" t="inlineStr">
-        <is>
-          <t>종합병원 전신마취치료비(급여, 4시간이상) — 6시간 이상이면 이 담보도 함께 지급된다(별개 특약 · 각각 제1조 충족)(v8.61)</t>
-        </is>
-      </c>
-      <c r="P99" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q99" s="10" t="inlineStr"/>
-      <c r="R99" s="10" t="inlineStr">
-        <is>
-          <t>종합병원 전신마취치료비 (급여, 4시간이상)
-종합병원 전신마취치료비 (급여, 4시간이상)</t>
-        </is>
-      </c>
       <c r="S99" s="11" t="inlineStr"/>
       <c r="T99" s="11" t="inlineStr"/>
     </row>
@@ -8488,7 +8506,7 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>tx_anesth</t>
+          <t>tx_anesth6</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
@@ -8498,14 +8516,10 @@
       </c>
       <c r="D100" s="13" t="inlineStr">
         <is>
-          <t>전신마취치료비</t>
-        </is>
-      </c>
-      <c r="E100" s="15" t="inlineStr">
-        <is>
-          <t>시간이상</t>
-        </is>
-      </c>
+          <t>전신마취치료비\(급여,6시간이상\)</t>
+        </is>
+      </c>
+      <c r="E100" s="15" t="inlineStr"/>
       <c r="F100" s="15" t="inlineStr">
         <is>
           <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
@@ -8523,7 +8537,7 @@
       </c>
       <c r="I100" s="15" t="inlineStr">
         <is>
-          <t>종합병원 전신마취 수술  (anes)</t>
+          <t>6시간 이상 전신마취 수술  (anes6)</t>
         </is>
       </c>
       <c r="J100" s="15" t="inlineStr"/>
@@ -8536,12 +8550,12 @@
       </c>
       <c r="N100" s="15" t="inlineStr">
         <is>
-          <t>종합병원 전신마취 · 치료 1회당</t>
+          <t>종합병원 전신마취 6시간 이상 · 치료 1회당</t>
         </is>
       </c>
       <c r="O100" s="15" t="inlineStr">
         <is>
-          <t>종합병원 전신마취치료비(급여) — 마취시간 조건 없음 · 치료 1회당 · 수가코드 L1211·L1221·L1231·L1212·L1222·L1232(제3조) · 제5조③ 면책질병은 db.json x 로 판정(v8.61 : 예전엔 acts anes6 만 보고 있어 사례가 anes6 를 주지 않아 0원이었다)</t>
+          <t>종합병원 전신마취치료비(급여, 6시간이상) — 약관 제1조 '전신마취치료(급여)를 6시간 이상 받은 때 치료 1회당' · 제2조① 마취시간은 1회당 기준(합산 없음) · 연간 횟수 제한 없음(v8.61)</t>
         </is>
       </c>
       <c r="P100" s="12" t="n">
@@ -8550,8 +8564,8 @@
       <c r="Q100" s="15" t="inlineStr"/>
       <c r="R100" s="15" t="inlineStr">
         <is>
-          <t>종합병원 전신마취치료비(급여)
-종합병원 전신마취치료비(급여)</t>
+          <t>종합병원 전신마취치료비 (급여, 6시간이상)
+종합병원 전신마취치료비 (급여, 6시간이상)</t>
         </is>
       </c>
       <c r="S100" s="11" t="inlineStr"/>
@@ -8563,7 +8577,7 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>tx_rehab</t>
+          <t>tx_anesth4</t>
         </is>
       </c>
       <c r="C101" s="9" t="inlineStr">
@@ -8573,7 +8587,7 @@
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>재활치료비</t>
+          <t>전신마취치료비\(급여,4시간이상\)</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr"/>
@@ -8594,7 +8608,7 @@
       </c>
       <c r="I101" s="10" t="inlineStr">
         <is>
-          <t>재활치료  (rehab)</t>
+          <t>4시간 이상 전신마취 수술  (anes4)</t>
         </is>
       </c>
       <c r="J101" s="10" t="inlineStr"/>
@@ -8607,21 +8621,22 @@
       </c>
       <c r="N101" s="10" t="inlineStr">
         <is>
-          <t>재활치료</t>
+          <t>종합병원 전신마취 4시간 이상 · 치료 1회당</t>
         </is>
       </c>
       <c r="O101" s="10" t="inlineStr">
         <is>
-          <t>재활치료비</t>
+          <t>종합병원 전신마취치료비(급여, 4시간이상) — 6시간 이상이면 이 담보도 함께 지급된다(별개 특약 · 각각 제1조 충족)(v8.61)</t>
         </is>
       </c>
       <c r="P101" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q101" s="10" t="inlineStr"/>
       <c r="R101" s="10" t="inlineStr">
         <is>
-          <t>상해재활치료비 (급여,1일1회한,연간15회한)</t>
+          <t>종합병원 전신마취치료비 (급여, 4시간이상)
+종합병원 전신마취치료비 (급여, 4시간이상)</t>
         </is>
       </c>
       <c r="S101" s="11" t="inlineStr"/>
@@ -8633,36 +8648,181 @@
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
+          <t>tx_anesth</t>
+        </is>
+      </c>
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D102" s="13" t="inlineStr">
+        <is>
+          <t>전신마취치료비</t>
+        </is>
+      </c>
+      <c r="E102" s="15" t="inlineStr">
+        <is>
+          <t>시간이상</t>
+        </is>
+      </c>
+      <c r="F102" s="15" t="inlineStr">
+        <is>
+          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
+        </is>
+      </c>
+      <c r="G102" s="12" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H102" s="12" t="inlineStr">
+        <is>
+          <t>받을 때마다</t>
+        </is>
+      </c>
+      <c r="I102" s="15" t="inlineStr">
+        <is>
+          <t>종합병원 전신마취 수술  (anes)</t>
+        </is>
+      </c>
+      <c r="J102" s="15" t="inlineStr"/>
+      <c r="K102" s="15" t="inlineStr"/>
+      <c r="L102" s="15" t="inlineStr"/>
+      <c r="M102" s="15" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N102" s="15" t="inlineStr">
+        <is>
+          <t>종합병원 전신마취 · 치료 1회당</t>
+        </is>
+      </c>
+      <c r="O102" s="15" t="inlineStr">
+        <is>
+          <t>종합병원 전신마취치료비(급여) — 마취시간 조건 없음 · 치료 1회당 · 수가코드 L1211·L1221·L1231·L1212·L1222·L1232(제3조) · 제5조③ 면책질병은 db.json x 로 판정(v8.61 : 예전엔 acts anes6 만 보고 있어 사례가 anes6 를 주지 않아 0원이었다)</t>
+        </is>
+      </c>
+      <c r="P102" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q102" s="15" t="inlineStr"/>
+      <c r="R102" s="15" t="inlineStr">
+        <is>
+          <t>종합병원 전신마취치료비(급여)
+종합병원 전신마취치료비(급여)</t>
+        </is>
+      </c>
+      <c r="S102" s="11" t="inlineStr"/>
+      <c r="T102" s="11" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="7" t="n">
+        <v>101</v>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>tx_rehab</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>재활치료비</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr"/>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
+          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
+        </is>
+      </c>
+      <c r="G103" s="7" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H103" s="7" t="inlineStr">
+        <is>
+          <t>받을 때마다</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t>재활치료  (rehab)</t>
+        </is>
+      </c>
+      <c r="J103" s="10" t="inlineStr"/>
+      <c r="K103" s="10" t="inlineStr"/>
+      <c r="L103" s="10" t="inlineStr"/>
+      <c r="M103" s="10" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N103" s="10" t="inlineStr">
+        <is>
+          <t>재활치료</t>
+        </is>
+      </c>
+      <c r="O103" s="10" t="inlineStr">
+        <is>
+          <t>재활치료비</t>
+        </is>
+      </c>
+      <c r="P103" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q103" s="10" t="inlineStr"/>
+      <c r="R103" s="10" t="inlineStr">
+        <is>
+          <t>상해재활치료비 (급여,1일1회한,연간15회한)</t>
+        </is>
+      </c>
+      <c r="S103" s="11" t="inlineStr"/>
+      <c r="T103" s="11" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="12" t="n">
+        <v>102</v>
+      </c>
+      <c r="B104" s="13" t="inlineStr">
+        <is>
           <t>tx_exam</t>
         </is>
       </c>
-      <c r="C102" s="14" t="inlineStr">
+      <c r="C104" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D102" s="13" t="inlineStr">
+      <c r="D104" s="13" t="inlineStr">
         <is>
           <t>(MRI|CT|PET|양전자단층촬영|초음파|내시경|NGS유전자|생검).*(검사비|촬영검사비)</t>
         </is>
       </c>
-      <c r="E102" s="15" t="inlineStr"/>
-      <c r="F102" s="15" t="inlineStr">
+      <c r="E104" s="15" t="inlineStr"/>
+      <c r="F104" s="15" t="inlineStr">
         <is>
           <t>마스터에 약관 KCD 목록이 있으면 대조 (없으면 조건 없이 계산하고 로그)</t>
         </is>
       </c>
-      <c r="G102" s="12" t="inlineStr">
+      <c r="G104" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H102" s="12" t="inlineStr">
+      <c r="H104" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I102" s="15" t="inlineStr">
+      <c r="I104" s="15" t="inlineStr">
         <is>
           <t>CT 검사  (x_ct)
 MRI 검사  (x_mri)
@@ -8673,153 +8833,6 @@
 조직검사(생검)  (x_bio)</t>
         </is>
       </c>
-      <c r="J102" s="15" t="inlineStr"/>
-      <c r="K102" s="15" t="inlineStr"/>
-      <c r="L102" s="15" t="inlineStr"/>
-      <c r="M102" s="15" t="inlineStr">
-        <is>
-          <t>치료비</t>
-        </is>
-      </c>
-      <c r="N102" s="15" t="inlineStr">
-        <is>
-          <t>검사 · 연간 1회</t>
-        </is>
-      </c>
-      <c r="O102" s="15" t="inlineStr">
-        <is>
-          <t>검사비 — 약관이 대상 질병을 정해 둔 담보(3대질환 MRI촬영검사비 등)는 마스터의 약관 KCD 목록과 대조한다. 목록이 없는 담보는 질병 조건 없이 계산하고 로그를 남긴다(v8.53)</t>
-        </is>
-      </c>
-      <c r="P102" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q102" s="15" t="inlineStr"/>
-      <c r="R102" s="15" t="inlineStr">
-        <is>
-          <t>갱신형 3대질환 MRI촬영검사비(급여, 연간1회한)
-갱신형 양전자단층촬영(PET)검사비(급여, 연간1회한)
-상해MRI/CT검사비 (급여,연간1회한)</t>
-        </is>
-      </c>
-      <c r="S102" s="11" t="inlineStr"/>
-      <c r="T102" s="11" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="7" t="n">
-        <v>101</v>
-      </c>
-      <c r="B103" s="8" t="inlineStr">
-        <is>
-          <t>tx_procedure</t>
-        </is>
-      </c>
-      <c r="C103" s="9" t="inlineStr">
-        <is>
-          <t>치료비 (치료행위)</t>
-        </is>
-      </c>
-      <c r="D103" s="8" t="inlineStr">
-        <is>
-          <t>(체외충격파쇄석술|신경차단술|고주파열치료|특정급여시술치료비|특정이물제거|창상봉합술|견봉성형술|특정비급여,신의료기술치료비|특정질환3대치료비|통합외상치료비|특정치료비)</t>
-        </is>
-      </c>
-      <c r="E103" s="10" t="inlineStr"/>
-      <c r="F103" s="10" t="inlineStr">
-        <is>
-          <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
-        </is>
-      </c>
-      <c r="G103" s="7" t="inlineStr">
-        <is>
-          <t>계산함</t>
-        </is>
-      </c>
-      <c r="H103" s="7" t="inlineStr">
-        <is>
-          <t>연 1회</t>
-        </is>
-      </c>
-      <c r="I103" s="10" t="inlineStr">
-        <is>
-          <t>수술  (surg)</t>
-        </is>
-      </c>
-      <c r="J103" s="10" t="inlineStr"/>
-      <c r="K103" s="10" t="inlineStr"/>
-      <c r="L103" s="10" t="inlineStr">
-        <is>
-          <t>약관이 진료행위(수가)코드를 열거한 항목은 그 목록에 있을 때만</t>
-        </is>
-      </c>
-      <c r="M103" s="10" t="inlineStr">
-        <is>
-          <t>치료비</t>
-        </is>
-      </c>
-      <c r="N103" s="10" t="inlineStr">
-        <is>
-          <t>약관 대상 시술 · 연간 1회</t>
-        </is>
-      </c>
-      <c r="O103" s="10" t="inlineStr">
-        <is>
-          <t>특정 시술·치료비</t>
-        </is>
-      </c>
-      <c r="P103" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q103" s="10" t="inlineStr"/>
-      <c r="R103" s="10" t="inlineStr">
-        <is>
-          <t>추간판장애(디스크질환) 신경차단술치료비(급여,연간1회한)
-특정이물제거치료비Ⅰ(급여,연간1회한)</t>
-        </is>
-      </c>
-      <c r="S103" s="11" t="inlineStr"/>
-      <c r="T103" s="11" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="12" t="n">
-        <v>102</v>
-      </c>
-      <c r="B104" s="13" t="inlineStr">
-        <is>
-          <t>tx_emergency</t>
-        </is>
-      </c>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>치료비 (치료행위)</t>
-        </is>
-      </c>
-      <c r="D104" s="13" t="inlineStr">
-        <is>
-          <t>응급실내원비</t>
-        </is>
-      </c>
-      <c r="E104" s="15" t="inlineStr"/>
-      <c r="F104" s="15" t="inlineStr">
-        <is>
-          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
-        </is>
-      </c>
-      <c r="G104" s="12" t="inlineStr">
-        <is>
-          <t>계산함</t>
-        </is>
-      </c>
-      <c r="H104" s="12" t="inlineStr">
-        <is>
-          <t>받을 때마다</t>
-        </is>
-      </c>
-      <c r="I104" s="15" t="inlineStr">
-        <is>
-          <t>응급실 진료  (er)</t>
-        </is>
-      </c>
       <c r="J104" s="15" t="inlineStr"/>
       <c r="K104" s="15" t="inlineStr"/>
       <c r="L104" s="15" t="inlineStr"/>
@@ -8830,19 +8843,166 @@
       </c>
       <c r="N104" s="15" t="inlineStr">
         <is>
-          <t>응급실 내원</t>
+          <t>검사 · 연간 1회</t>
         </is>
       </c>
       <c r="O104" s="15" t="inlineStr">
         <is>
-          <t>응급실 내원비</t>
+          <t>검사비 — 약관이 대상 질병을 정해 둔 담보(3대질환 MRI촬영검사비 등)는 마스터의 약관 KCD 목록과 대조한다. 목록이 없는 담보는 질병 조건 없이 계산하고 로그를 남긴다(v8.53)</t>
         </is>
       </c>
       <c r="P104" s="12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q104" s="15" t="inlineStr"/>
       <c r="R104" s="15" t="inlineStr">
+        <is>
+          <t>갱신형 3대질환 MRI촬영검사비(급여, 연간1회한)
+갱신형 양전자단층촬영(PET)검사비(급여, 연간1회한)
+상해MRI/CT검사비 (급여,연간1회한)</t>
+        </is>
+      </c>
+      <c r="S104" s="11" t="inlineStr"/>
+      <c r="T104" s="11" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="n">
+        <v>103</v>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>tx_procedure</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>(체외충격파쇄석술|신경차단술|고주파열치료|특정급여시술치료비|특정이물제거|창상봉합술|견봉성형술|특정비급여,신의료기술치료비|특정질환3대치료비|통합외상치료비|특정치료비)</t>
+        </is>
+      </c>
+      <c r="E105" s="10" t="inlineStr"/>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
+          <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
+        </is>
+      </c>
+      <c r="G105" s="7" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>연 1회</t>
+        </is>
+      </c>
+      <c r="I105" s="10" t="inlineStr">
+        <is>
+          <t>수술  (surg)</t>
+        </is>
+      </c>
+      <c r="J105" s="10" t="inlineStr"/>
+      <c r="K105" s="10" t="inlineStr"/>
+      <c r="L105" s="10" t="inlineStr">
+        <is>
+          <t>약관이 진료행위(수가)코드를 열거한 항목은 그 목록에 있을 때만</t>
+        </is>
+      </c>
+      <c r="M105" s="10" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N105" s="10" t="inlineStr">
+        <is>
+          <t>약관 대상 시술 · 연간 1회</t>
+        </is>
+      </c>
+      <c r="O105" s="10" t="inlineStr">
+        <is>
+          <t>특정 시술·치료비</t>
+        </is>
+      </c>
+      <c r="P105" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q105" s="10" t="inlineStr"/>
+      <c r="R105" s="10" t="inlineStr">
+        <is>
+          <t>추간판장애(디스크질환) 신경차단술치료비(급여,연간1회한)
+특정이물제거치료비Ⅰ(급여,연간1회한)</t>
+        </is>
+      </c>
+      <c r="S105" s="11" t="inlineStr"/>
+      <c r="T105" s="11" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="12" t="n">
+        <v>104</v>
+      </c>
+      <c r="B106" s="13" t="inlineStr">
+        <is>
+          <t>tx_emergency</t>
+        </is>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>치료비 (치료행위)</t>
+        </is>
+      </c>
+      <c r="D106" s="13" t="inlineStr">
+        <is>
+          <t>응급실내원비</t>
+        </is>
+      </c>
+      <c r="E106" s="15" t="inlineStr"/>
+      <c r="F106" s="15" t="inlineStr">
+        <is>
+          <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
+        </is>
+      </c>
+      <c r="G106" s="12" t="inlineStr">
+        <is>
+          <t>계산함</t>
+        </is>
+      </c>
+      <c r="H106" s="12" t="inlineStr">
+        <is>
+          <t>받을 때마다</t>
+        </is>
+      </c>
+      <c r="I106" s="15" t="inlineStr">
+        <is>
+          <t>응급실 진료  (er)</t>
+        </is>
+      </c>
+      <c r="J106" s="15" t="inlineStr"/>
+      <c r="K106" s="15" t="inlineStr"/>
+      <c r="L106" s="15" t="inlineStr"/>
+      <c r="M106" s="15" t="inlineStr">
+        <is>
+          <t>치료비</t>
+        </is>
+      </c>
+      <c r="N106" s="15" t="inlineStr">
+        <is>
+          <t>응급실 내원</t>
+        </is>
+      </c>
+      <c r="O106" s="15" t="inlineStr">
+        <is>
+          <t>응급실 내원비</t>
+        </is>
+      </c>
+      <c r="P106" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q106" s="15" t="inlineStr"/>
+      <c r="R106" s="15" t="inlineStr">
         <is>
           <t>응급실내원비(응급)
 상해 응급실내원비(응급)
@@ -8851,60 +9011,60 @@
 의료기관 및 민간 구급차 이용 응급실내원비(1-3등급)</t>
         </is>
       </c>
-      <c r="S104" s="11" t="inlineStr"/>
-      <c r="T104" s="11" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="7" t="n">
-        <v>103</v>
-      </c>
-      <c r="B105" s="8" t="inlineStr">
+      <c r="S106" s="11" t="inlineStr"/>
+      <c r="T106" s="11" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="n">
+        <v>105</v>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
         <is>
           <t>ls_monthly</t>
         </is>
       </c>
-      <c r="C105" s="9" t="inlineStr">
+      <c r="C107" s="9" t="inlineStr">
         <is>
           <t>생활지원금</t>
         </is>
       </c>
-      <c r="D105" s="8" t="inlineStr">
+      <c r="D107" s="8" t="inlineStr">
         <is>
           <t>통합생활지원비</t>
         </is>
       </c>
-      <c r="E105" s="10" t="inlineStr"/>
-      <c r="F105" s="10" t="inlineStr">
+      <c r="E107" s="10" t="inlineStr"/>
+      <c r="F107" s="10" t="inlineStr">
         <is>
           <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
         </is>
       </c>
-      <c r="G105" s="7" t="inlineStr">
+      <c r="G107" s="7" t="inlineStr">
         <is>
           <t>분류만 (금액 계산 안 함)</t>
         </is>
       </c>
-      <c r="H105" s="7" t="inlineStr">
+      <c r="H107" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I105" s="10" t="inlineStr"/>
-      <c r="J105" s="10" t="inlineStr"/>
-      <c r="K105" s="10" t="inlineStr"/>
-      <c r="L105" s="10" t="inlineStr"/>
-      <c r="M105" s="10" t="inlineStr"/>
-      <c r="N105" s="10" t="inlineStr"/>
-      <c r="O105" s="10" t="inlineStr">
+      <c r="I107" s="10" t="inlineStr"/>
+      <c r="J107" s="10" t="inlineStr"/>
+      <c r="K107" s="10" t="inlineStr"/>
+      <c r="L107" s="10" t="inlineStr"/>
+      <c r="M107" s="10" t="inlineStr"/>
+      <c r="N107" s="10" t="inlineStr"/>
+      <c r="O107" s="10" t="inlineStr">
         <is>
           <t>통합생활지원비 — 산정특례 등록·치료 항목마다 월 단위 지급(가입금액 = 월간 총 지급금액 한도). 정액 치료비로 오계산되지 않게 사례 계산에서 제외하고, 약관 항목표(life_support.json)를 전용 지면에 그대로 싣는다.</t>
         </is>
       </c>
-      <c r="P105" s="7" t="n">
+      <c r="P107" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="Q105" s="10" t="inlineStr"/>
-      <c r="R105" s="10" t="inlineStr">
+      <c r="Q107" s="10" t="inlineStr"/>
+      <c r="R107" s="10" t="inlineStr">
         <is>
           <t>암 통합생활지원비(월간한도)
 2대질환 통합생활지원비(월간한도)
@@ -8913,142 +9073,142 @@
 상해 통합생활지원비(월간한도)</t>
         </is>
       </c>
-      <c r="S105" s="11" t="inlineStr"/>
-      <c r="T105" s="11" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="12" t="n">
-        <v>104</v>
-      </c>
-      <c r="B106" s="13" t="inlineStr">
+      <c r="S107" s="11" t="inlineStr"/>
+      <c r="T107" s="11" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="12" t="n">
+        <v>106</v>
+      </c>
+      <c r="B108" s="13" t="inlineStr">
         <is>
           <t>tx_aneurysm_surg</t>
         </is>
       </c>
-      <c r="C106" s="14" t="inlineStr">
+      <c r="C108" s="14" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D106" s="13" t="inlineStr">
+      <c r="D108" s="13" t="inlineStr">
         <is>
           <t>뇌동맥류수술비</t>
         </is>
       </c>
-      <c r="E106" s="15" t="inlineStr"/>
-      <c r="F106" s="15" t="inlineStr">
+      <c r="E108" s="15" t="inlineStr"/>
+      <c r="F108" s="15" t="inlineStr">
         <is>
           <t>질병코드 조건 없음 — 담보명·치료행위로만 판정</t>
         </is>
       </c>
-      <c r="G106" s="12" t="inlineStr">
+      <c r="G108" s="12" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H106" s="12" t="inlineStr">
+      <c r="H108" s="12" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I106" s="15" t="inlineStr">
+      <c r="I108" s="15" t="inlineStr">
         <is>
           <t>수술  (surg)</t>
         </is>
       </c>
-      <c r="J106" s="15" t="inlineStr"/>
-      <c r="K106" s="15" t="inlineStr"/>
-      <c r="L106" s="15" t="inlineStr">
+      <c r="J108" s="15" t="inlineStr"/>
+      <c r="K108" s="15" t="inlineStr"/>
+      <c r="L108" s="15" t="inlineStr">
         <is>
           <t>1-7종 분류표의 수술구분이 「뇌동맥류수술」일 때만</t>
         </is>
       </c>
-      <c r="M106" s="15" t="inlineStr">
+      <c r="M108" s="15" t="inlineStr">
         <is>
           <t>수술비</t>
         </is>
       </c>
-      <c r="N106" s="15" t="inlineStr">
+      <c r="N108" s="15" t="inlineStr">
         <is>
           <t>뇌동맥류수술(약관 별표 1-7종 수술분류표 「뇌동맥류수술」 B011~B018) · 연간 1회</t>
         </is>
       </c>
-      <c r="O106" s="15" t="inlineStr">
+      <c r="O108" s="15" t="inlineStr">
         <is>
           <t>뇌동맥류수술비 — 약관 별표 1-7종 수술분류표의 수술구분 「뇌동맥류수술」에 드는 수술을 받은 단계에서만 지급. 대상 질병(파열되지 않은 대뇌동맥의 박리·파열되지 않은 뇌동맥류)은 이 상품 약관 별표가 있어야 코드로 가릴 수 있어, 지금은 그 병을 다루는 사례(뇌동맥류(미파열) 코일 색전술)에서만 계산한다.</t>
         </is>
       </c>
-      <c r="P106" s="16" t="n">
+      <c r="P108" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="Q106" s="17" t="inlineStr">
+      <c r="Q108" s="17" t="inlineStr">
         <is>
           <t>특약 마스터에 이 담보명이 없음 — 상품에 없는 담보이거나 이름이 달라진 것</t>
         </is>
       </c>
-      <c r="R106" s="15" t="inlineStr"/>
-      <c r="S106" s="11" t="inlineStr"/>
-      <c r="T106" s="11" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="7" t="n">
-        <v>105</v>
-      </c>
-      <c r="B107" s="8" t="inlineStr">
+      <c r="R108" s="15" t="inlineStr"/>
+      <c r="S108" s="11" t="inlineStr"/>
+      <c r="T108" s="11" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="n">
+        <v>107</v>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
         <is>
           <t>tx_etc_care</t>
         </is>
       </c>
-      <c r="C107" s="9" t="inlineStr">
+      <c r="C109" s="9" t="inlineStr">
         <is>
           <t>치료비 (치료행위)</t>
         </is>
       </c>
-      <c r="D107" s="8" t="inlineStr">
+      <c r="D109" s="8" t="inlineStr">
         <is>
           <t>치료비|생활비|생활지원비|지원금|입원비|검사비|대기등록</t>
         </is>
       </c>
-      <c r="E107" s="10" t="inlineStr"/>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="E109" s="10" t="inlineStr"/>
+      <c r="F109" s="10" t="inlineStr">
         <is>
           <t>특약 마스터(db.json)에 실린 약관 KCD 목록과 대조</t>
         </is>
       </c>
-      <c r="G107" s="7" t="inlineStr">
+      <c r="G109" s="7" t="inlineStr">
         <is>
           <t>계산함</t>
         </is>
       </c>
-      <c r="H107" s="7" t="inlineStr">
+      <c r="H109" s="7" t="inlineStr">
         <is>
           <t>연 1회</t>
         </is>
       </c>
-      <c r="I107" s="10" t="inlineStr"/>
-      <c r="J107" s="10" t="inlineStr"/>
-      <c r="K107" s="10" t="inlineStr"/>
-      <c r="L107" s="10" t="inlineStr"/>
-      <c r="M107" s="10" t="inlineStr">
+      <c r="I109" s="10" t="inlineStr"/>
+      <c r="J109" s="10" t="inlineStr"/>
+      <c r="K109" s="10" t="inlineStr"/>
+      <c r="L109" s="10" t="inlineStr"/>
+      <c r="M109" s="10" t="inlineStr">
         <is>
           <t>치료비</t>
         </is>
       </c>
-      <c r="N107" s="10" t="inlineStr">
+      <c r="N109" s="10" t="inlineStr">
         <is>
           <t>약관 대상 치료</t>
         </is>
       </c>
-      <c r="O107" s="10" t="inlineStr">
+      <c r="O109" s="10" t="inlineStr">
         <is>
           <t>그 밖의 치료비 — 약관 KCD 목록이 있을 때만 판정</t>
         </is>
       </c>
-      <c r="P107" s="7" t="n">
+      <c r="P109" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="Q107" s="10" t="inlineStr"/>
-      <c r="R107" s="10" t="inlineStr">
+      <c r="Q109" s="10" t="inlineStr"/>
+      <c r="R109" s="10" t="inlineStr">
         <is>
           <t>갱신형 영구치상실치료비
 갱신형 치석제거(스케일링)치료비
@@ -9056,13 +9216,13 @@
 갱신형 치면열구전색술(실란트)치료비</t>
         </is>
       </c>
-      <c r="S107" s="11" t="inlineStr"/>
-      <c r="T107" s="11" t="inlineStr"/>
+      <c r="S109" s="11" t="inlineStr"/>
+      <c r="T109" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:T107"/>
+  <autoFilter ref="A2:T109"/>
   <dataValidations count="1">
-    <dataValidation sqref="S3:S107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="검수 결과" prompt="O = 약관과 맞음 / X = 고쳐야 함 / 보류 = 확인 필요" type="list">
+    <dataValidation sqref="S3:S109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="검수 결과" prompt="O = 약관과 맞음 / X = 고쳐야 함 / 보류 = 확인 필요" type="list">
       <formula1>"O,X,보류"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9129,11 +9289,11 @@
         </is>
       </c>
       <c r="C7" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B7&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B7&amp;"*")</f>
         <v/>
       </c>
       <c r="D7" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B7&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B7&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9144,11 +9304,11 @@
         </is>
       </c>
       <c r="C8" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B8&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B8&amp;"*")</f>
         <v/>
       </c>
       <c r="D8" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B8&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B8&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9159,11 +9319,11 @@
         </is>
       </c>
       <c r="C9" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B9&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B9&amp;"*")</f>
         <v/>
       </c>
       <c r="D9" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B9&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B9&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9174,11 +9334,11 @@
         </is>
       </c>
       <c r="C10" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B10&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B10&amp;"*")</f>
         <v/>
       </c>
       <c r="D10" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B10&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B10&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9189,11 +9349,11 @@
         </is>
       </c>
       <c r="C11" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B11&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B11&amp;"*")</f>
         <v/>
       </c>
       <c r="D11" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B11&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B11&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9204,11 +9364,11 @@
         </is>
       </c>
       <c r="C12" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B12&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B12&amp;"*")</f>
         <v/>
       </c>
       <c r="D12" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B12&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B12&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9219,11 +9379,11 @@
         </is>
       </c>
       <c r="C13" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B13&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B13&amp;"*")</f>
         <v/>
       </c>
       <c r="D13" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B13&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B13&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9234,11 +9394,11 @@
         </is>
       </c>
       <c r="C14" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B14&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B14&amp;"*")</f>
         <v/>
       </c>
       <c r="D14" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B14&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B14&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9249,11 +9409,11 @@
         </is>
       </c>
       <c r="C15" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B15&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B15&amp;"*")</f>
         <v/>
       </c>
       <c r="D15" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B15&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B15&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9264,11 +9424,11 @@
         </is>
       </c>
       <c r="C16" s="23">
-        <f>COUNTIF('규칙 105개'!C3:C107,B16&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!C3:C109,B16&amp;"*")</f>
         <v/>
       </c>
       <c r="D16" s="23">
-        <f>SUMIF('규칙 105개'!C3:C107,B16&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!C3:C109,B16&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9318,11 +9478,11 @@
         </is>
       </c>
       <c r="C21" s="23">
-        <f>COUNTIF('규칙 105개'!H3:H107,B21&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!H3:H109,B21&amp;"*")</f>
         <v/>
       </c>
       <c r="D21" s="23">
-        <f>SUMIF('규칙 105개'!H3:H107,B21&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!H3:H109,B21&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9333,11 +9493,11 @@
         </is>
       </c>
       <c r="C22" s="23">
-        <f>COUNTIF('규칙 105개'!H3:H107,B22&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!H3:H109,B22&amp;"*")</f>
         <v/>
       </c>
       <c r="D22" s="23">
-        <f>SUMIF('규칙 105개'!H3:H107,B22&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!H3:H109,B22&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9348,11 +9508,11 @@
         </is>
       </c>
       <c r="C23" s="23">
-        <f>COUNTIF('규칙 105개'!H3:H107,B23&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!H3:H109,B23&amp;"*")</f>
         <v/>
       </c>
       <c r="D23" s="23">
-        <f>SUMIF('규칙 105개'!H3:H107,B23&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!H3:H109,B23&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9363,11 +9523,11 @@
         </is>
       </c>
       <c r="C24" s="23">
-        <f>COUNTIF('규칙 105개'!H3:H107,B24&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!H3:H109,B24&amp;"*")</f>
         <v/>
       </c>
       <c r="D24" s="23">
-        <f>SUMIF('규칙 105개'!H3:H107,B24&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!H3:H109,B24&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9417,11 +9577,11 @@
         </is>
       </c>
       <c r="C29" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B29&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B29&amp;"*")</f>
         <v/>
       </c>
       <c r="D29" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B29&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B29&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9432,11 +9592,11 @@
         </is>
       </c>
       <c r="C30" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B30&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B30&amp;"*")</f>
         <v/>
       </c>
       <c r="D30" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B30&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B30&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9447,11 +9607,11 @@
         </is>
       </c>
       <c r="C31" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B31&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B31&amp;"*")</f>
         <v/>
       </c>
       <c r="D31" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B31&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B31&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9462,11 +9622,11 @@
         </is>
       </c>
       <c r="C32" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B32&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B32&amp;"*")</f>
         <v/>
       </c>
       <c r="D32" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B32&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B32&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9477,11 +9637,11 @@
         </is>
       </c>
       <c r="C33" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B33&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B33&amp;"*")</f>
         <v/>
       </c>
       <c r="D33" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B33&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B33&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9492,11 +9652,11 @@
         </is>
       </c>
       <c r="C34" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B34&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B34&amp;"*")</f>
         <v/>
       </c>
       <c r="D34" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B34&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B34&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9507,11 +9667,11 @@
         </is>
       </c>
       <c r="C35" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B35&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B35&amp;"*")</f>
         <v/>
       </c>
       <c r="D35" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B35&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B35&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>
@@ -9522,11 +9682,11 @@
         </is>
       </c>
       <c r="C36" s="23">
-        <f>COUNTIF('규칙 105개'!F3:F107,B36&amp;"*")</f>
+        <f>COUNTIF('규칙 107개'!F3:F109,B36&amp;"*")</f>
         <v/>
       </c>
       <c r="D36" s="23">
-        <f>SUMIF('규칙 105개'!F3:F107,B36&amp;"*",'규칙 105개'!$P$3:$P$107)</f>
+        <f>SUMIF('규칙 107개'!F3:F109,B36&amp;"*",'규칙 107개'!$P$3:$P$109)</f>
         <v/>
       </c>
     </row>

</xml_diff>